<commit_message>
Dashboard update 2026-08-02 09:39
</commit_message>
<xml_diff>
--- a/excel/Investavimas Rima.xlsx
+++ b/excel/Investavimas Rima.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.06.03\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evald\OneDrive\Dokumentai\portfolio-analytics\portfolio-dashboard-clean\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8B64DB0-C519-4F3A-A565-06D5D5BB689F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C034FA5-F525-430B-86E0-2AC3AD45975E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4109,80 +4109,80 @@
         <v>0</v>
       </c>
       <c r="AI19" s="4">
-        <f t="shared" ref="AI19" si="172">I19+L19+O19+R19+U19</f>
+        <f>I19+L19+O19+R19+U19</f>
         <v>2199.12</v>
       </c>
       <c r="AJ19" s="4">
-        <f t="shared" ref="AJ19" si="173">AI19-AG19</f>
+        <f t="shared" ref="AJ19" si="172">AI19-AG19</f>
         <v>244.76999999999998</v>
       </c>
       <c r="AK19" s="13">
-        <f t="shared" ref="AK19" si="174">AJ19/AG19</f>
+        <f t="shared" ref="AK19" si="173">AJ19/AG19</f>
         <v>0.12524368715941361</v>
       </c>
       <c r="AL19" s="4">
-        <f t="shared" ref="AL19" si="175">AJ19-AJ18</f>
+        <f t="shared" ref="AL19" si="174">AJ19-AJ18</f>
         <v>7.2399999999997817</v>
       </c>
       <c r="AM19" s="10"/>
       <c r="AN19" s="8">
-        <f t="shared" ref="AN19" si="176">A19</f>
+        <f t="shared" ref="AN19" si="175">A19</f>
         <v>46234</v>
       </c>
       <c r="AO19" s="4">
-        <f t="shared" ref="AO19" si="177">Y19+AG19</f>
+        <f t="shared" ref="AO19" si="176">Y19+AG19</f>
         <v>3194.35</v>
       </c>
       <c r="AP19" s="4">
-        <f t="shared" ref="AP19" si="178">AO19-AO18</f>
+        <f t="shared" ref="AP19" si="177">AO19-AO18</f>
         <v>130</v>
       </c>
       <c r="AQ19" s="4">
-        <f t="shared" ref="AQ19" si="179">AA19+AI19</f>
+        <f t="shared" ref="AQ19" si="178">AA19+AI19</f>
         <v>3536.99</v>
       </c>
       <c r="AR19" s="4">
-        <f t="shared" ref="AR19" si="180">AQ19-AO19</f>
+        <f t="shared" ref="AR19" si="179">AQ19-AO19</f>
         <v>342.63999999999987</v>
       </c>
       <c r="AS19" s="13">
-        <f t="shared" ref="AS19" si="181">AR19/AO19</f>
+        <f t="shared" ref="AS19" si="180">AR19/AO19</f>
         <v>0.10726438868627416</v>
       </c>
       <c r="AT19" s="4">
-        <f t="shared" ref="AT19" si="182">AR19-AR18</f>
+        <f t="shared" ref="AT19" si="181">AR19-AR18</f>
         <v>-1.4400000000005093</v>
       </c>
       <c r="AV19" s="8">
-        <f t="shared" ref="AV19" si="183">A19</f>
+        <f t="shared" ref="AV19" si="182">A19</f>
         <v>46234</v>
       </c>
       <c r="AW19" s="4">
-        <f t="shared" ref="AW19" si="184">(C19-B19)-(C18-B18)</f>
+        <f t="shared" ref="AW19" si="183">(C19-B19)-(C18-B18)</f>
         <v>2.2700000000000955</v>
       </c>
       <c r="AX19" s="4">
-        <f t="shared" ref="AX19" si="185">(F19-E19)-(F18-E18)</f>
+        <f t="shared" ref="AX19" si="184">(F19-E19)-(F18-E18)</f>
         <v>-10.950000000000045</v>
       </c>
       <c r="AY19" s="4">
-        <f t="shared" ref="AY19" si="186">(I19-H19)-(I18-H18)</f>
+        <f t="shared" ref="AY19" si="185">(I19-H19)-(I18-H18)</f>
         <v>0</v>
       </c>
       <c r="AZ19" s="4">
-        <f t="shared" ref="AZ19" si="187">(L19-K19)-(L18-K18)</f>
+        <f t="shared" ref="AZ19" si="186">(L19-K19)-(L18-K18)</f>
         <v>2.2400000000000091</v>
       </c>
       <c r="BA19" s="4">
-        <f t="shared" ref="BA19" si="188">(O19-N19)-(O18-N18)</f>
+        <f t="shared" ref="BA19" si="187">(O19-N19)-(O18-N18)</f>
         <v>2.5400000000000773</v>
       </c>
       <c r="BB19" s="4">
-        <f t="shared" ref="BB19" si="189">(R19-Q19)-(R18-Q18)</f>
+        <f t="shared" ref="BB19" si="188">(R19-Q19)-(R18-Q18)</f>
         <v>1.7599999999999909</v>
       </c>
       <c r="BC19" s="4">
-        <f t="shared" ref="BC19" si="190">(U19-T19)-(U18-T18)</f>
+        <f t="shared" ref="BC19" si="189">(U19-T19)-(U18-T18)</f>
         <v>0.69999999999998863</v>
       </c>
     </row>
@@ -4205,7 +4205,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="AP3:AP17" formula="1"/>
+    <ignoredError sqref="AP3:AP19" formula="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dashboard update 2026-08-07 20:13
</commit_message>
<xml_diff>
--- a/excel/Investavimas Rima.xlsx
+++ b/excel/Investavimas Rima.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evald\OneDrive\Dokumentai\portfolio-analytics\portfolio-dashboard-clean\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.06.03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C034FA5-F525-430B-86E0-2AC3AD45975E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1A73A3A-DD42-4CEB-A3E9-8CE2945A1E9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="18">
   <si>
     <t>Data</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>Viso</t>
+  </si>
+  <si>
+    <t>Debitum</t>
   </si>
 </sst>
 </file>
@@ -295,7 +298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -348,6 +351,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -685,93 +691,99 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BD19"/>
+  <dimension ref="A1:BH19"/>
   <sheetFormatPr defaultColWidth="10.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="5" max="7" width="10.7109375" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:56" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="25" t="s">
+    <row r="1" spans="1:60" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25" t="s">
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25" t="s">
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25" t="s">
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25" t="s">
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="O1" s="25"/>
-      <c r="P1" s="25"/>
-      <c r="Q1" s="25" t="s">
+      <c r="O1" s="26"/>
+      <c r="P1" s="26"/>
+      <c r="Q1" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="R1" s="25"/>
-      <c r="S1" s="25"/>
-      <c r="T1" s="25" t="s">
+      <c r="R1" s="26"/>
+      <c r="S1" s="26"/>
+      <c r="T1" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="U1" s="25"/>
-      <c r="V1" s="25"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="26" t="s">
+      <c r="U1" s="26"/>
+      <c r="V1" s="26"/>
+      <c r="W1" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="X1" s="26"/>
+      <c r="Y1" s="26"/>
+      <c r="Z1" s="3"/>
+      <c r="AA1" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="Y1" s="26"/>
-      <c r="Z1" s="26"/>
-      <c r="AA1" s="26"/>
-      <c r="AB1" s="26"/>
-      <c r="AC1" s="26"/>
-      <c r="AD1" s="26"/>
-      <c r="AE1" s="3"/>
-      <c r="AF1" s="26" t="s">
+      <c r="AB1" s="27"/>
+      <c r="AC1" s="27"/>
+      <c r="AD1" s="27"/>
+      <c r="AE1" s="27"/>
+      <c r="AF1" s="27"/>
+      <c r="AG1" s="27"/>
+      <c r="AH1" s="3"/>
+      <c r="AI1" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="AG1" s="26"/>
-      <c r="AH1" s="26"/>
-      <c r="AI1" s="26"/>
-      <c r="AJ1" s="26"/>
-      <c r="AK1" s="26"/>
-      <c r="AL1" s="26"/>
-      <c r="AM1" s="17"/>
-      <c r="AN1" s="26" t="s">
+      <c r="AJ1" s="27"/>
+      <c r="AK1" s="27"/>
+      <c r="AL1" s="27"/>
+      <c r="AM1" s="27"/>
+      <c r="AN1" s="27"/>
+      <c r="AO1" s="27"/>
+      <c r="AP1" s="17"/>
+      <c r="AQ1" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="AO1" s="26"/>
-      <c r="AP1" s="26"/>
-      <c r="AQ1" s="26"/>
-      <c r="AR1" s="26"/>
-      <c r="AS1" s="26"/>
-      <c r="AT1" s="26"/>
-      <c r="AU1" s="18"/>
-      <c r="AV1" s="20"/>
-      <c r="AW1" s="21"/>
-      <c r="AX1" s="21"/>
+      <c r="AR1" s="27"/>
+      <c r="AS1" s="27"/>
+      <c r="AT1" s="27"/>
+      <c r="AU1" s="27"/>
+      <c r="AV1" s="27"/>
+      <c r="AW1" s="27"/>
+      <c r="AX1" s="18"/>
       <c r="AY1" s="21"/>
-      <c r="AZ1" s="21"/>
-      <c r="BA1" s="21"/>
-      <c r="BB1" s="21"/>
+      <c r="AZ1" s="22"/>
+      <c r="BA1" s="22"/>
+      <c r="BB1" s="22"/>
       <c r="BC1" s="22"/>
+      <c r="BD1" s="22"/>
+      <c r="BE1" s="22"/>
+      <c r="BF1" s="22"/>
+      <c r="BG1" s="23"/>
     </row>
-    <row r="2" spans="1:56" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="24"/>
+    <row r="2" spans="1:60" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="25"/>
       <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
@@ -826,115 +838,128 @@
       <c r="S2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="T2" s="7" t="s">
+      <c r="T2" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="U2" s="7" t="s">
+      <c r="U2" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="V2" s="7" t="s">
+      <c r="V2" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="W2" s="3"/>
-      <c r="X2" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="Y2" s="15" t="s">
+      <c r="W2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="Z2" s="15" t="s">
+      <c r="X2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="Y2" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="Z2" s="3"/>
+      <c r="AA2" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="AB2" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="AA2" s="15" t="s">
+      <c r="AD2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="AB2" s="15" t="s">
+      <c r="AE2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="AC2" s="15" t="s">
+      <c r="AF2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="AD2" s="15" t="s">
+      <c r="AG2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="AE2" s="17"/>
-      <c r="AF2" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="AG2" s="15" t="s">
+      <c r="AH2" s="17"/>
+      <c r="AI2" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="AJ2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="AH2" s="15" t="s">
+      <c r="AK2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="AI2" s="15" t="s">
+      <c r="AL2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="AJ2" s="15" t="s">
+      <c r="AM2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="AK2" s="15" t="s">
+      <c r="AN2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="AL2" s="15" t="s">
+      <c r="AO2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="AM2" s="17"/>
-      <c r="AN2" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="AO2" s="15" t="s">
+      <c r="AP2" s="17"/>
+      <c r="AQ2" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="AR2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="AP2" s="15" t="s">
+      <c r="AS2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="AQ2" s="15" t="s">
+      <c r="AT2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="AR2" s="15" t="s">
+      <c r="AU2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="AS2" s="15" t="s">
+      <c r="AV2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="AT2" s="15" t="s">
+      <c r="AW2" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="AV2" s="7" t="str">
+      <c r="AY2" s="7" t="str">
         <f>A1</f>
         <v>Data</v>
       </c>
-      <c r="AW2" s="7" t="str">
+      <c r="AZ2" s="7" t="str">
         <f>B1</f>
         <v>SEB Fondai</v>
       </c>
-      <c r="AX2" s="7" t="str">
+      <c r="BA2" s="7" t="str">
         <f>E1</f>
         <v>Revolut Brokerage</v>
       </c>
-      <c r="AY2" s="7" t="str">
+      <c r="BB2" s="7" t="str">
         <f>H1</f>
         <v>Indemo</v>
       </c>
-      <c r="AZ2" s="7" t="str">
+      <c r="BC2" s="7" t="str">
         <f>K1</f>
         <v>Profitus</v>
       </c>
-      <c r="BA2" s="7" t="str">
+      <c r="BD2" s="7" t="str">
         <f>N1</f>
         <v>Nordstreet</v>
       </c>
-      <c r="BB2" s="7" t="str">
+      <c r="BE2" s="7" t="str">
         <f>Q1</f>
         <v>Scramble</v>
       </c>
-      <c r="BC2" s="16" t="str">
+      <c r="BF2" s="16" t="str">
         <f>T1</f>
         <v>Lendermarket</v>
       </c>
+      <c r="BG2" s="16" t="str">
+        <f>W1</f>
+        <v>Debitum</v>
+      </c>
     </row>
-    <row r="3" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>45747</v>
       </c>
@@ -1003,127 +1028,140 @@
       <c r="V3" s="12">
         <v>0</v>
       </c>
-      <c r="W3" s="10"/>
-      <c r="X3" s="8">
+      <c r="W3" s="5">
+        <v>0</v>
+      </c>
+      <c r="X3" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="12">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="10"/>
+      <c r="AA3" s="8">
         <f>A3</f>
         <v>45747</v>
       </c>
-      <c r="Y3" s="4">
+      <c r="AB3" s="4">
         <f>B3+E3</f>
         <v>60</v>
       </c>
-      <c r="Z3" s="4">
-        <f>Y3</f>
+      <c r="AC3" s="4">
+        <f>AB3</f>
         <v>60</v>
       </c>
-      <c r="AA3" s="4">
+      <c r="AD3" s="4">
         <f>C3+F3</f>
         <v>58.94</v>
       </c>
-      <c r="AB3" s="4">
-        <f t="shared" ref="AB3" si="1">AA3-Y3</f>
+      <c r="AE3" s="4">
+        <f t="shared" ref="AE3" si="1">AD3-AB3</f>
         <v>-1.0600000000000023</v>
       </c>
-      <c r="AC3" s="13">
-        <f t="shared" ref="AC3" si="2">AB3/Y3</f>
+      <c r="AF3" s="13">
+        <f t="shared" ref="AF3" si="2">AE3/AB3</f>
         <v>-1.7666666666666705E-2</v>
       </c>
-      <c r="AD3" s="4">
-        <f>AB3</f>
+      <c r="AG3" s="4">
+        <f>AE3</f>
         <v>-1.0600000000000023</v>
       </c>
-      <c r="AE3" s="10"/>
-      <c r="AF3" s="8">
+      <c r="AH3" s="10"/>
+      <c r="AI3" s="8">
         <f>A3</f>
         <v>45747</v>
       </c>
-      <c r="AG3" s="4">
-        <f>H3+K3+N3+Q3+T3</f>
+      <c r="AJ3" s="4">
+        <f>H3+K3+N3+Q3+T3+W3</f>
         <v>10</v>
       </c>
-      <c r="AH3" s="4">
-        <f>AG3</f>
+      <c r="AK3" s="4">
+        <f>AJ3</f>
         <v>10</v>
       </c>
-      <c r="AI3" s="4">
-        <f>I3+L3+O3+R3+U3</f>
+      <c r="AL3" s="4">
+        <f>I3+L3+O3+R3+U3+X3</f>
         <v>65</v>
       </c>
-      <c r="AJ3" s="4">
-        <f t="shared" ref="AJ3:AJ16" si="3">AI3-AG3</f>
+      <c r="AM3" s="4">
+        <f t="shared" ref="AM3:AM16" si="3">AL3-AJ3</f>
         <v>55</v>
       </c>
-      <c r="AK3" s="13">
-        <f t="shared" ref="AK3:AK16" si="4">AJ3/AG3</f>
+      <c r="AN3" s="13">
+        <f t="shared" ref="AN3:AN16" si="4">AM3/AJ3</f>
         <v>5.5</v>
       </c>
-      <c r="AL3" s="4">
-        <f>AJ3</f>
+      <c r="AO3" s="4">
+        <f>AM3</f>
         <v>55</v>
       </c>
-      <c r="AM3" s="10"/>
-      <c r="AN3" s="8">
+      <c r="AP3" s="10"/>
+      <c r="AQ3" s="8">
         <f>A3</f>
         <v>45747</v>
       </c>
-      <c r="AO3" s="4">
-        <f>Y3+AG3</f>
+      <c r="AR3" s="4">
+        <f>AB3+AJ3</f>
         <v>70</v>
       </c>
-      <c r="AP3" s="4">
-        <f>AO3</f>
+      <c r="AS3" s="4">
+        <f>AR3</f>
         <v>70</v>
       </c>
-      <c r="AQ3" s="4">
-        <f>AA3+AI3</f>
+      <c r="AT3" s="4">
+        <f>AD3+AL3</f>
         <v>123.94</v>
       </c>
-      <c r="AR3" s="4">
-        <f t="shared" ref="AR3:AR16" si="5">AQ3-AO3</f>
+      <c r="AU3" s="4">
+        <f t="shared" ref="AU3:AU16" si="5">AT3-AR3</f>
         <v>53.94</v>
       </c>
-      <c r="AS3" s="13">
-        <f t="shared" ref="AS3:AS16" si="6">AR3/AO3</f>
+      <c r="AV3" s="13">
+        <f t="shared" ref="AV3:AV16" si="6">AU3/AR3</f>
         <v>0.77057142857142857</v>
       </c>
-      <c r="AT3" s="4">
-        <f>AR3</f>
+      <c r="AW3" s="4">
+        <f>AU3</f>
         <v>53.94</v>
       </c>
-      <c r="AV3" s="14">
-        <f t="shared" ref="AV3:AV14" si="7">A3</f>
+      <c r="AY3" s="14">
+        <f t="shared" ref="AY3:AY14" si="7">A3</f>
         <v>45747</v>
       </c>
-      <c r="AW3" s="6">
+      <c r="AZ3" s="6">
         <f>(C3-B3)</f>
         <v>-1.0600000000000023</v>
       </c>
-      <c r="AX3" s="6">
+      <c r="BA3" s="6">
         <f>(F3-E3)</f>
         <v>0</v>
       </c>
-      <c r="AY3" s="6">
+      <c r="BB3" s="6">
         <f>(I3-H3)</f>
         <v>55</v>
       </c>
-      <c r="AZ3" s="6">
+      <c r="BC3" s="6">
         <f>(L3-K3)</f>
         <v>0</v>
       </c>
-      <c r="BA3" s="6">
+      <c r="BD3" s="6">
         <f>(O3-N3)</f>
         <v>0</v>
       </c>
-      <c r="BB3" s="6">
+      <c r="BE3" s="6">
         <f>(R3-Q3)</f>
         <v>0</v>
       </c>
-      <c r="BC3" s="6">
+      <c r="BF3" s="6">
         <f>(U3-T3)</f>
         <v>0</v>
       </c>
+      <c r="BG3" s="6">
+        <f>(X3-W3)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>45777</v>
       </c>
@@ -1192,127 +1230,140 @@
       <c r="V4" s="12">
         <v>0</v>
       </c>
-      <c r="W4" s="10"/>
-      <c r="X4" s="8">
-        <f t="shared" ref="X4:X14" si="9">A4</f>
+      <c r="W4" s="5">
+        <v>0</v>
+      </c>
+      <c r="X4" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="12">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="10"/>
+      <c r="AA4" s="8">
+        <f t="shared" ref="AA4:AA14" si="9">A4</f>
         <v>45777</v>
       </c>
-      <c r="Y4" s="4">
-        <f t="shared" ref="Y4:Y16" si="10">B4+E4</f>
+      <c r="AB4" s="4">
+        <f t="shared" ref="AB4:AB16" si="10">B4+E4</f>
         <v>90</v>
       </c>
-      <c r="Z4" s="4">
-        <f>Y4-Y3</f>
+      <c r="AC4" s="4">
+        <f>AB4-AB3</f>
         <v>30</v>
       </c>
-      <c r="AA4" s="4">
-        <f t="shared" ref="AA4:AA16" si="11">C4+F4</f>
+      <c r="AD4" s="4">
+        <f t="shared" ref="AD4:AD16" si="11">C4+F4</f>
         <v>87.26</v>
       </c>
-      <c r="AB4" s="4">
-        <f t="shared" ref="AB4:AB14" si="12">AA4-Y4</f>
+      <c r="AE4" s="4">
+        <f t="shared" ref="AE4:AE14" si="12">AD4-AB4</f>
         <v>-2.7399999999999949</v>
       </c>
-      <c r="AC4" s="13">
-        <f t="shared" ref="AC4:AC14" si="13">AB4/Y4</f>
+      <c r="AF4" s="13">
+        <f t="shared" ref="AF4:AF14" si="13">AE4/AB4</f>
         <v>-3.0444444444444389E-2</v>
       </c>
-      <c r="AD4" s="4">
-        <f>AB4-AB3</f>
+      <c r="AG4" s="4">
+        <f>AE4-AE3</f>
         <v>-1.6799999999999926</v>
       </c>
-      <c r="AE4" s="10"/>
-      <c r="AF4" s="8">
-        <f t="shared" ref="AF4:AF16" si="14">A4</f>
+      <c r="AH4" s="10"/>
+      <c r="AI4" s="8">
+        <f t="shared" ref="AI4:AI16" si="14">A4</f>
         <v>45777</v>
       </c>
-      <c r="AG4" s="4">
-        <f t="shared" ref="AG4:AG16" si="15">H4+K4+N4+Q4+T4</f>
+      <c r="AJ4" s="4">
+        <f t="shared" ref="AJ4:AJ19" si="15">H4+K4+N4+Q4+T4+W4</f>
         <v>10</v>
       </c>
-      <c r="AH4" s="4">
-        <f>AG4-AG3</f>
-        <v>0</v>
-      </c>
-      <c r="AI4" s="4">
-        <f t="shared" ref="AI4:AI16" si="16">I4+L4+O4+R4+U4</f>
+      <c r="AK4" s="4">
+        <f>AJ4-AJ3</f>
+        <v>0</v>
+      </c>
+      <c r="AL4" s="4">
+        <f t="shared" ref="AL4:AL19" si="16">I4+L4+O4+R4+U4+X4</f>
         <v>65</v>
       </c>
-      <c r="AJ4" s="4">
+      <c r="AM4" s="4">
         <f t="shared" si="3"/>
         <v>55</v>
       </c>
-      <c r="AK4" s="13">
+      <c r="AN4" s="13">
         <f t="shared" si="4"/>
         <v>5.5</v>
       </c>
-      <c r="AL4" s="4">
-        <f>AJ4-AJ3</f>
-        <v>0</v>
-      </c>
-      <c r="AM4" s="10"/>
-      <c r="AN4" s="8">
-        <f t="shared" ref="AN4:AN16" si="17">A4</f>
+      <c r="AO4" s="4">
+        <f>AM4-AM3</f>
+        <v>0</v>
+      </c>
+      <c r="AP4" s="10"/>
+      <c r="AQ4" s="8">
+        <f t="shared" ref="AQ4:AQ16" si="17">A4</f>
         <v>45777</v>
       </c>
-      <c r="AO4" s="4">
-        <f t="shared" ref="AO4:AO16" si="18">Y4+AG4</f>
+      <c r="AR4" s="4">
+        <f t="shared" ref="AR4:AR16" si="18">AB4+AJ4</f>
         <v>100</v>
       </c>
-      <c r="AP4" s="4">
-        <f>AO4-AO3</f>
+      <c r="AS4" s="4">
+        <f>AR4-AR3</f>
         <v>30</v>
       </c>
-      <c r="AQ4" s="4">
-        <f t="shared" ref="AQ4:AQ16" si="19">AA4+AI4</f>
+      <c r="AT4" s="4">
+        <f t="shared" ref="AT4:AT16" si="19">AD4+AL4</f>
         <v>152.26</v>
       </c>
-      <c r="AR4" s="4">
+      <c r="AU4" s="4">
         <f t="shared" si="5"/>
         <v>52.259999999999991</v>
       </c>
-      <c r="AS4" s="13">
+      <c r="AV4" s="13">
         <f t="shared" si="6"/>
         <v>0.52259999999999995</v>
       </c>
-      <c r="AT4" s="4">
-        <f>AR4-AR3</f>
+      <c r="AW4" s="4">
+        <f>AU4-AU3</f>
         <v>-1.6800000000000068</v>
       </c>
-      <c r="AV4" s="8">
+      <c r="AY4" s="8">
         <f t="shared" si="7"/>
         <v>45777</v>
       </c>
-      <c r="AW4" s="4">
-        <f t="shared" ref="AW4:AW14" si="20">(C4-B4)-(C3-B3)</f>
+      <c r="AZ4" s="4">
+        <f t="shared" ref="AZ4:AZ14" si="20">(C4-B4)-(C3-B3)</f>
         <v>-1.6799999999999926</v>
       </c>
-      <c r="AX4" s="4">
-        <f t="shared" ref="AX4:AX14" si="21">(F4-E4)-(F3-E3)</f>
-        <v>0</v>
-      </c>
-      <c r="AY4" s="4">
-        <f t="shared" ref="AY4:AY14" si="22">(I4-H4)-(I3-H3)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ4" s="4">
-        <f t="shared" ref="AZ4:AZ14" si="23">(L4-K4)-(L3-K3)</f>
-        <v>0</v>
-      </c>
       <c r="BA4" s="4">
-        <f t="shared" ref="BA4:BA14" si="24">(O4-N4)-(O3-N3)</f>
+        <f t="shared" ref="BA4:BA14" si="21">(F4-E4)-(F3-E3)</f>
         <v>0</v>
       </c>
       <c r="BB4" s="4">
-        <f t="shared" ref="BB4:BB14" si="25">(R4-Q4)-(R3-Q3)</f>
+        <f t="shared" ref="BB4:BB14" si="22">(I4-H4)-(I3-H3)</f>
         <v>0</v>
       </c>
       <c r="BC4" s="4">
+        <f t="shared" ref="BC4:BC14" si="23">(L4-K4)-(L3-K3)</f>
+        <v>0</v>
+      </c>
+      <c r="BD4" s="4">
+        <f t="shared" ref="BD4:BD14" si="24">(O4-N4)-(O3-N3)</f>
+        <v>0</v>
+      </c>
+      <c r="BE4" s="4">
+        <f t="shared" ref="BE4:BE14" si="25">(R4-Q4)-(R3-Q3)</f>
+        <v>0</v>
+      </c>
+      <c r="BF4" s="4">
         <f>(U4-T4)-(U3-T3)</f>
         <v>0</v>
       </c>
+      <c r="BG4" s="4">
+        <f>(X4-W4)-(X3-W3)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>45808</v>
       </c>
@@ -1381,127 +1432,140 @@
       <c r="V5" s="12">
         <v>0</v>
       </c>
-      <c r="W5" s="10"/>
-      <c r="X5" s="8">
+      <c r="W5" s="5">
+        <v>0</v>
+      </c>
+      <c r="X5" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="12">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="10"/>
+      <c r="AA5" s="8">
         <f t="shared" si="9"/>
         <v>45808</v>
       </c>
-      <c r="Y5" s="4">
+      <c r="AB5" s="4">
         <f t="shared" si="10"/>
         <v>120</v>
       </c>
-      <c r="Z5" s="4">
-        <f t="shared" ref="Z5:Z16" si="26">Y5-Y4</f>
+      <c r="AC5" s="4">
+        <f t="shared" ref="AC5:AC16" si="26">AB5-AB4</f>
         <v>30</v>
       </c>
-      <c r="AA5" s="4">
+      <c r="AD5" s="4">
         <f t="shared" si="11"/>
         <v>121.7</v>
       </c>
-      <c r="AB5" s="4">
+      <c r="AE5" s="4">
         <f t="shared" si="12"/>
         <v>1.7000000000000028</v>
       </c>
-      <c r="AC5" s="13">
+      <c r="AF5" s="13">
         <f t="shared" si="13"/>
         <v>1.416666666666669E-2</v>
       </c>
-      <c r="AD5" s="4">
-        <f t="shared" ref="AD5:AD14" si="27">AB5-AB4</f>
+      <c r="AG5" s="4">
+        <f t="shared" ref="AG5:AG14" si="27">AE5-AE4</f>
         <v>4.4399999999999977</v>
       </c>
-      <c r="AE5" s="10"/>
-      <c r="AF5" s="8">
+      <c r="AH5" s="10"/>
+      <c r="AI5" s="8">
         <f t="shared" si="14"/>
         <v>45808</v>
       </c>
-      <c r="AG5" s="4">
+      <c r="AJ5" s="4">
         <f t="shared" si="15"/>
         <v>10</v>
       </c>
-      <c r="AH5" s="4">
-        <f t="shared" ref="AH5:AH16" si="28">AG5-AG4</f>
-        <v>0</v>
-      </c>
-      <c r="AI5" s="4">
+      <c r="AK5" s="4">
+        <f t="shared" ref="AK5:AK16" si="28">AJ5-AJ4</f>
+        <v>0</v>
+      </c>
+      <c r="AL5" s="4">
         <f t="shared" si="16"/>
         <v>65</v>
       </c>
-      <c r="AJ5" s="4">
+      <c r="AM5" s="4">
         <f t="shared" si="3"/>
         <v>55</v>
       </c>
-      <c r="AK5" s="13">
+      <c r="AN5" s="13">
         <f t="shared" si="4"/>
         <v>5.5</v>
       </c>
-      <c r="AL5" s="4">
-        <f t="shared" ref="AL5:AL16" si="29">AJ5-AJ4</f>
-        <v>0</v>
-      </c>
-      <c r="AM5" s="10"/>
-      <c r="AN5" s="8">
+      <c r="AO5" s="4">
+        <f t="shared" ref="AO5:AO16" si="29">AM5-AM4</f>
+        <v>0</v>
+      </c>
+      <c r="AP5" s="10"/>
+      <c r="AQ5" s="8">
         <f t="shared" si="17"/>
         <v>45808</v>
       </c>
-      <c r="AO5" s="4">
+      <c r="AR5" s="4">
         <f t="shared" si="18"/>
         <v>130</v>
       </c>
-      <c r="AP5" s="4">
-        <f t="shared" ref="AP5:AP16" si="30">AO5-AO4</f>
+      <c r="AS5" s="4">
+        <f t="shared" ref="AS5:AS16" si="30">AR5-AR4</f>
         <v>30</v>
       </c>
-      <c r="AQ5" s="4">
+      <c r="AT5" s="4">
         <f t="shared" si="19"/>
         <v>186.7</v>
       </c>
-      <c r="AR5" s="4">
+      <c r="AU5" s="4">
         <f t="shared" si="5"/>
         <v>56.699999999999989</v>
       </c>
-      <c r="AS5" s="13">
+      <c r="AV5" s="13">
         <f t="shared" si="6"/>
         <v>0.43615384615384606</v>
       </c>
-      <c r="AT5" s="4">
-        <f t="shared" ref="AT5:AT16" si="31">AR5-AR4</f>
+      <c r="AW5" s="4">
+        <f t="shared" ref="AW5:AW16" si="31">AU5-AU4</f>
         <v>4.4399999999999977</v>
       </c>
-      <c r="AV5" s="8">
+      <c r="AY5" s="8">
         <f t="shared" si="7"/>
         <v>45808</v>
       </c>
-      <c r="AW5" s="4">
+      <c r="AZ5" s="4">
         <f t="shared" si="20"/>
         <v>4.4399999999999977</v>
       </c>
-      <c r="AX5" s="4">
+      <c r="BA5" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="AY5" s="4">
+      <c r="BB5" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="AZ5" s="4">
+      <c r="BC5" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="BA5" s="4">
+      <c r="BD5" s="4">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="BB5" s="4">
+      <c r="BE5" s="4">
         <f t="shared" si="25"/>
         <v>0</v>
       </c>
-      <c r="BC5" s="4">
-        <f t="shared" ref="BC5:BC15" si="32">(U5-T5)-(U4-T4)</f>
+      <c r="BF5" s="4">
+        <f t="shared" ref="BF5:BF19" si="32">(U5-T5)-(U4-T4)</f>
+        <v>0</v>
+      </c>
+      <c r="BG5" s="4">
+        <f t="shared" ref="BF5:BG15" si="33">(X5-W5)-(X4-W4)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>45838</v>
       </c>
@@ -1570,127 +1634,140 @@
       <c r="V6" s="12">
         <v>0</v>
       </c>
-      <c r="W6" s="10"/>
-      <c r="X6" s="8">
+      <c r="W6" s="5">
+        <v>0</v>
+      </c>
+      <c r="X6" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y6" s="12">
+        <v>0</v>
+      </c>
+      <c r="Z6" s="10"/>
+      <c r="AA6" s="8">
         <f t="shared" si="9"/>
         <v>45838</v>
       </c>
-      <c r="Y6" s="4">
+      <c r="AB6" s="4">
         <f t="shared" si="10"/>
         <v>150</v>
       </c>
-      <c r="Z6" s="4">
+      <c r="AC6" s="4">
         <f t="shared" si="26"/>
         <v>30</v>
       </c>
-      <c r="AA6" s="4">
+      <c r="AD6" s="4">
         <f t="shared" si="11"/>
         <v>151.65</v>
       </c>
-      <c r="AB6" s="4">
+      <c r="AE6" s="4">
         <f t="shared" si="12"/>
         <v>1.6500000000000057</v>
       </c>
-      <c r="AC6" s="13">
+      <c r="AF6" s="13">
         <f t="shared" si="13"/>
         <v>1.1000000000000038E-2</v>
       </c>
-      <c r="AD6" s="4">
+      <c r="AG6" s="4">
         <f t="shared" si="27"/>
         <v>-4.9999999999997158E-2</v>
       </c>
-      <c r="AE6" s="10"/>
-      <c r="AF6" s="8">
+      <c r="AH6" s="10"/>
+      <c r="AI6" s="8">
         <f t="shared" si="14"/>
         <v>45838</v>
       </c>
-      <c r="AG6" s="4">
+      <c r="AJ6" s="4">
         <f t="shared" si="15"/>
         <v>30</v>
       </c>
-      <c r="AH6" s="4">
+      <c r="AK6" s="4">
         <f t="shared" si="28"/>
         <v>20</v>
       </c>
-      <c r="AI6" s="4">
+      <c r="AL6" s="4">
         <f t="shared" si="16"/>
         <v>85.05</v>
       </c>
-      <c r="AJ6" s="4">
+      <c r="AM6" s="4">
         <f t="shared" si="3"/>
         <v>55.05</v>
       </c>
-      <c r="AK6" s="13">
+      <c r="AN6" s="13">
         <f t="shared" si="4"/>
         <v>1.835</v>
       </c>
-      <c r="AL6" s="4">
+      <c r="AO6" s="4">
         <f t="shared" si="29"/>
         <v>4.9999999999997158E-2</v>
       </c>
-      <c r="AM6" s="10"/>
-      <c r="AN6" s="8">
+      <c r="AP6" s="10"/>
+      <c r="AQ6" s="8">
         <f t="shared" si="17"/>
         <v>45838</v>
       </c>
-      <c r="AO6" s="4">
+      <c r="AR6" s="4">
         <f t="shared" si="18"/>
         <v>180</v>
       </c>
-      <c r="AP6" s="4">
+      <c r="AS6" s="4">
         <f t="shared" si="30"/>
         <v>50</v>
       </c>
-      <c r="AQ6" s="4">
+      <c r="AT6" s="4">
         <f t="shared" si="19"/>
         <v>236.7</v>
       </c>
-      <c r="AR6" s="4">
+      <c r="AU6" s="4">
         <f t="shared" si="5"/>
         <v>56.699999999999989</v>
       </c>
-      <c r="AS6" s="13">
+      <c r="AV6" s="13">
         <f t="shared" si="6"/>
         <v>0.31499999999999995</v>
       </c>
-      <c r="AT6" s="4">
+      <c r="AW6" s="4">
         <f t="shared" si="31"/>
         <v>0</v>
       </c>
-      <c r="AV6" s="8">
+      <c r="AY6" s="8">
         <f t="shared" si="7"/>
         <v>45838</v>
       </c>
-      <c r="AW6" s="4">
+      <c r="AZ6" s="4">
         <f t="shared" si="20"/>
         <v>-4.9999999999997158E-2</v>
       </c>
-      <c r="AX6" s="4">
+      <c r="BA6" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="AY6" s="4">
+      <c r="BB6" s="4">
         <f t="shared" si="22"/>
         <v>4.9999999999997158E-2</v>
       </c>
-      <c r="AZ6" s="4">
+      <c r="BC6" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="BA6" s="4">
+      <c r="BD6" s="4">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="BB6" s="4">
+      <c r="BE6" s="4">
         <f t="shared" si="25"/>
         <v>0</v>
       </c>
-      <c r="BC6" s="4">
+      <c r="BF6" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
+      <c r="BG6" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>45869</v>
       </c>
@@ -1759,127 +1836,140 @@
       <c r="V7" s="12">
         <v>0</v>
       </c>
-      <c r="W7" s="10"/>
-      <c r="X7" s="8">
+      <c r="W7" s="5">
+        <v>0</v>
+      </c>
+      <c r="X7" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y7" s="12">
+        <v>0</v>
+      </c>
+      <c r="Z7" s="10"/>
+      <c r="AA7" s="8">
         <f t="shared" si="9"/>
         <v>45869</v>
       </c>
-      <c r="Y7" s="4">
+      <c r="AB7" s="4">
         <f t="shared" si="10"/>
         <v>180</v>
       </c>
-      <c r="Z7" s="4">
+      <c r="AC7" s="4">
         <f t="shared" si="26"/>
         <v>30</v>
       </c>
-      <c r="AA7" s="4">
+      <c r="AD7" s="4">
         <f t="shared" si="11"/>
         <v>184.1</v>
       </c>
-      <c r="AB7" s="4">
+      <c r="AE7" s="4">
         <f t="shared" si="12"/>
         <v>4.0999999999999943</v>
       </c>
-      <c r="AC7" s="13">
+      <c r="AF7" s="13">
         <f t="shared" si="13"/>
         <v>2.2777777777777748E-2</v>
       </c>
-      <c r="AD7" s="4">
+      <c r="AG7" s="4">
         <f t="shared" si="27"/>
         <v>2.4499999999999886</v>
       </c>
-      <c r="AE7" s="10"/>
-      <c r="AF7" s="8">
+      <c r="AH7" s="10"/>
+      <c r="AI7" s="8">
         <f t="shared" si="14"/>
         <v>45869</v>
       </c>
-      <c r="AG7" s="4">
+      <c r="AJ7" s="4">
         <f t="shared" si="15"/>
         <v>30</v>
       </c>
-      <c r="AH7" s="4">
+      <c r="AK7" s="4">
         <f t="shared" si="28"/>
         <v>0</v>
       </c>
-      <c r="AI7" s="4">
+      <c r="AL7" s="4">
         <f t="shared" si="16"/>
         <v>85.05</v>
       </c>
-      <c r="AJ7" s="4">
+      <c r="AM7" s="4">
         <f t="shared" si="3"/>
         <v>55.05</v>
       </c>
-      <c r="AK7" s="13">
+      <c r="AN7" s="13">
         <f t="shared" si="4"/>
         <v>1.835</v>
       </c>
-      <c r="AL7" s="4">
+      <c r="AO7" s="4">
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
-      <c r="AM7" s="10"/>
-      <c r="AN7" s="8">
+      <c r="AP7" s="10"/>
+      <c r="AQ7" s="8">
         <f t="shared" si="17"/>
         <v>45869</v>
       </c>
-      <c r="AO7" s="4">
+      <c r="AR7" s="4">
         <f t="shared" si="18"/>
         <v>210</v>
       </c>
-      <c r="AP7" s="4">
+      <c r="AS7" s="4">
         <f t="shared" si="30"/>
         <v>30</v>
       </c>
-      <c r="AQ7" s="4">
+      <c r="AT7" s="4">
         <f t="shared" si="19"/>
         <v>269.14999999999998</v>
       </c>
-      <c r="AR7" s="4">
+      <c r="AU7" s="4">
         <f t="shared" si="5"/>
         <v>59.149999999999977</v>
       </c>
-      <c r="AS7" s="13">
+      <c r="AV7" s="13">
         <f t="shared" si="6"/>
         <v>0.28166666666666657</v>
       </c>
-      <c r="AT7" s="4">
+      <c r="AW7" s="4">
         <f t="shared" si="31"/>
         <v>2.4499999999999886</v>
       </c>
-      <c r="AV7" s="8">
+      <c r="AY7" s="8">
         <f t="shared" si="7"/>
         <v>45869</v>
       </c>
-      <c r="AW7" s="4">
+      <c r="AZ7" s="4">
         <f t="shared" si="20"/>
         <v>2.4499999999999886</v>
       </c>
-      <c r="AX7" s="4">
+      <c r="BA7" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="AY7" s="4">
+      <c r="BB7" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="AZ7" s="4">
+      <c r="BC7" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="BA7" s="4">
+      <c r="BD7" s="4">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="BB7" s="4">
+      <c r="BE7" s="4">
         <f t="shared" si="25"/>
         <v>0</v>
       </c>
-      <c r="BC7" s="4">
+      <c r="BF7" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
+      <c r="BG7" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>45900</v>
       </c>
@@ -1919,7 +2009,7 @@
         <v>400</v>
       </c>
       <c r="M8" s="12">
-        <f t="shared" ref="M8:M11" si="33">(L8-K8)/K8</f>
+        <f t="shared" ref="M8:M11" si="34">(L8-K8)/K8</f>
         <v>0</v>
       </c>
       <c r="N8" s="5">
@@ -1938,7 +2028,7 @@
         <v>430</v>
       </c>
       <c r="S8" s="12">
-        <f t="shared" ref="S8:S12" si="34">(R8-Q8)/Q8</f>
+        <f t="shared" ref="S8:S12" si="35">(R8-Q8)/Q8</f>
         <v>4.878048780487805E-2</v>
       </c>
       <c r="T8" s="5">
@@ -1950,127 +2040,140 @@
       <c r="V8" s="12">
         <v>0</v>
       </c>
-      <c r="W8" s="10"/>
-      <c r="X8" s="8">
+      <c r="W8" s="5">
+        <v>0</v>
+      </c>
+      <c r="X8" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="12">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="10"/>
+      <c r="AA8" s="8">
         <f t="shared" si="9"/>
         <v>45900</v>
       </c>
-      <c r="Y8" s="4">
+      <c r="AB8" s="4">
         <f t="shared" si="10"/>
         <v>210</v>
       </c>
-      <c r="Z8" s="4">
+      <c r="AC8" s="4">
         <f t="shared" si="26"/>
         <v>30</v>
       </c>
-      <c r="AA8" s="4">
+      <c r="AD8" s="4">
         <f t="shared" si="11"/>
         <v>214.63</v>
       </c>
-      <c r="AB8" s="4">
+      <c r="AE8" s="4">
         <f t="shared" si="12"/>
         <v>4.6299999999999955</v>
       </c>
-      <c r="AC8" s="13">
+      <c r="AF8" s="13">
         <f t="shared" si="13"/>
         <v>2.2047619047619024E-2</v>
       </c>
-      <c r="AD8" s="4">
+      <c r="AG8" s="4">
         <f t="shared" si="27"/>
         <v>0.53000000000000114</v>
       </c>
-      <c r="AE8" s="10"/>
-      <c r="AF8" s="8">
+      <c r="AH8" s="10"/>
+      <c r="AI8" s="8">
         <f t="shared" si="14"/>
         <v>45900</v>
       </c>
-      <c r="AG8" s="4">
+      <c r="AJ8" s="4">
         <f t="shared" si="15"/>
         <v>840</v>
       </c>
-      <c r="AH8" s="4">
+      <c r="AK8" s="4">
         <f t="shared" si="28"/>
         <v>810</v>
       </c>
-      <c r="AI8" s="4">
+      <c r="AL8" s="4">
         <f t="shared" si="16"/>
         <v>915.05</v>
       </c>
-      <c r="AJ8" s="4">
+      <c r="AM8" s="4">
         <f t="shared" si="3"/>
         <v>75.049999999999955</v>
       </c>
-      <c r="AK8" s="13">
+      <c r="AN8" s="13">
         <f t="shared" si="4"/>
         <v>8.9345238095238047E-2</v>
       </c>
-      <c r="AL8" s="4">
+      <c r="AO8" s="4">
         <f t="shared" si="29"/>
         <v>19.999999999999957</v>
       </c>
-      <c r="AM8" s="10"/>
-      <c r="AN8" s="8">
+      <c r="AP8" s="10"/>
+      <c r="AQ8" s="8">
         <f t="shared" si="17"/>
         <v>45900</v>
       </c>
-      <c r="AO8" s="4">
+      <c r="AR8" s="4">
         <f t="shared" si="18"/>
         <v>1050</v>
       </c>
-      <c r="AP8" s="4">
+      <c r="AS8" s="4">
         <f t="shared" si="30"/>
         <v>840</v>
       </c>
-      <c r="AQ8" s="4">
+      <c r="AT8" s="4">
         <f t="shared" si="19"/>
         <v>1129.6799999999998</v>
       </c>
-      <c r="AR8" s="4">
+      <c r="AU8" s="4">
         <f t="shared" si="5"/>
         <v>79.679999999999836</v>
       </c>
-      <c r="AS8" s="13">
+      <c r="AV8" s="13">
         <f t="shared" si="6"/>
         <v>7.5885714285714126E-2</v>
       </c>
-      <c r="AT8" s="4">
+      <c r="AW8" s="4">
         <f t="shared" si="31"/>
         <v>20.529999999999859</v>
       </c>
-      <c r="AV8" s="8">
+      <c r="AY8" s="8">
         <f t="shared" si="7"/>
         <v>45900</v>
       </c>
-      <c r="AW8" s="4">
+      <c r="AZ8" s="4">
         <f t="shared" si="20"/>
         <v>0.53000000000000114</v>
       </c>
-      <c r="AX8" s="4">
+      <c r="BA8" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="AY8" s="4">
+      <c r="BB8" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="AZ8" s="4">
+      <c r="BC8" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="BA8" s="4">
+      <c r="BD8" s="4">
         <f t="shared" si="24"/>
         <v>0</v>
       </c>
-      <c r="BB8" s="4">
+      <c r="BE8" s="4">
         <f t="shared" si="25"/>
         <v>20</v>
       </c>
-      <c r="BC8" s="4">
+      <c r="BF8" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
+      <c r="BG8" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>45930</v>
       </c>
@@ -2110,7 +2213,7 @@
         <v>400</v>
       </c>
       <c r="M9" s="12">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="N9" s="5">
@@ -2120,7 +2223,7 @@
         <v>401.7</v>
       </c>
       <c r="P9" s="12">
-        <f t="shared" ref="P9:P11" si="35">(O9-N9)/N9</f>
+        <f t="shared" ref="P9:P11" si="36">(O9-N9)/N9</f>
         <v>4.2499999999999717E-3</v>
       </c>
       <c r="Q9" s="5">
@@ -2130,7 +2233,7 @@
         <v>632</v>
       </c>
       <c r="S9" s="12">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>3.6065573770491806E-2</v>
       </c>
       <c r="T9" s="5">
@@ -2142,127 +2245,140 @@
       <c r="V9" s="12">
         <v>0</v>
       </c>
-      <c r="W9" s="10"/>
-      <c r="X9" s="8">
+      <c r="W9" s="5">
+        <v>0</v>
+      </c>
+      <c r="X9" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="12">
+        <v>0</v>
+      </c>
+      <c r="Z9" s="10"/>
+      <c r="AA9" s="8">
         <f t="shared" si="9"/>
         <v>45930</v>
       </c>
-      <c r="Y9" s="4">
+      <c r="AB9" s="4">
         <f t="shared" si="10"/>
         <v>240</v>
       </c>
-      <c r="Z9" s="4">
+      <c r="AC9" s="4">
         <f t="shared" si="26"/>
         <v>30</v>
       </c>
-      <c r="AA9" s="4">
+      <c r="AD9" s="4">
         <f t="shared" si="11"/>
         <v>246.01</v>
       </c>
-      <c r="AB9" s="4">
+      <c r="AE9" s="4">
         <f t="shared" si="12"/>
         <v>6.0099999999999909</v>
       </c>
-      <c r="AC9" s="13">
+      <c r="AF9" s="13">
         <f t="shared" si="13"/>
         <v>2.5041666666666629E-2</v>
       </c>
-      <c r="AD9" s="4">
+      <c r="AG9" s="4">
         <f t="shared" si="27"/>
         <v>1.3799999999999955</v>
       </c>
-      <c r="AE9" s="10"/>
-      <c r="AF9" s="8">
+      <c r="AH9" s="10"/>
+      <c r="AI9" s="8">
         <f t="shared" si="14"/>
         <v>45930</v>
       </c>
-      <c r="AG9" s="4">
+      <c r="AJ9" s="4">
         <f t="shared" si="15"/>
         <v>1440</v>
       </c>
-      <c r="AH9" s="4">
+      <c r="AK9" s="4">
         <f t="shared" si="28"/>
         <v>600</v>
       </c>
-      <c r="AI9" s="4">
+      <c r="AL9" s="4">
         <f t="shared" si="16"/>
         <v>1518.75</v>
       </c>
-      <c r="AJ9" s="4">
+      <c r="AM9" s="4">
         <f t="shared" si="3"/>
         <v>78.75</v>
       </c>
-      <c r="AK9" s="13">
+      <c r="AN9" s="13">
         <f t="shared" si="4"/>
         <v>5.46875E-2</v>
       </c>
-      <c r="AL9" s="4">
+      <c r="AO9" s="4">
         <f t="shared" si="29"/>
         <v>3.7000000000000455</v>
       </c>
-      <c r="AM9" s="10"/>
-      <c r="AN9" s="8">
+      <c r="AP9" s="10"/>
+      <c r="AQ9" s="8">
         <f t="shared" si="17"/>
         <v>45930</v>
       </c>
-      <c r="AO9" s="4">
+      <c r="AR9" s="4">
         <f t="shared" si="18"/>
         <v>1680</v>
       </c>
-      <c r="AP9" s="4">
+      <c r="AS9" s="4">
         <f t="shared" si="30"/>
         <v>630</v>
       </c>
-      <c r="AQ9" s="4">
+      <c r="AT9" s="4">
         <f t="shared" si="19"/>
         <v>1764.76</v>
       </c>
-      <c r="AR9" s="4">
+      <c r="AU9" s="4">
         <f t="shared" si="5"/>
         <v>84.759999999999991</v>
       </c>
-      <c r="AS9" s="13">
+      <c r="AV9" s="13">
         <f t="shared" si="6"/>
         <v>5.045238095238095E-2</v>
       </c>
-      <c r="AT9" s="4">
+      <c r="AW9" s="4">
         <f t="shared" si="31"/>
         <v>5.0800000000001546</v>
       </c>
-      <c r="AV9" s="8">
+      <c r="AY9" s="8">
         <f t="shared" si="7"/>
         <v>45930</v>
       </c>
-      <c r="AW9" s="4">
+      <c r="AZ9" s="4">
         <f t="shared" si="20"/>
         <v>1.3799999999999955</v>
       </c>
-      <c r="AX9" s="4">
+      <c r="BA9" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="AY9" s="4">
+      <c r="BB9" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="AZ9" s="4">
+      <c r="BC9" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="BA9" s="4">
+      <c r="BD9" s="4">
         <f t="shared" si="24"/>
         <v>1.6999999999999886</v>
       </c>
-      <c r="BB9" s="4">
+      <c r="BE9" s="4">
         <f t="shared" si="25"/>
         <v>2</v>
       </c>
-      <c r="BC9" s="4">
+      <c r="BF9" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
+      <c r="BG9" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>45961</v>
       </c>
@@ -2302,7 +2418,7 @@
         <v>400</v>
       </c>
       <c r="M10" s="12">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>0</v>
       </c>
       <c r="N10" s="5">
@@ -2312,7 +2428,7 @@
         <v>450.97</v>
       </c>
       <c r="P10" s="12">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>7.3738095238095297E-2</v>
       </c>
       <c r="Q10" s="5">
@@ -2322,7 +2438,7 @@
         <v>634</v>
       </c>
       <c r="S10" s="12">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>3.9344262295081971E-2</v>
       </c>
       <c r="T10" s="5">
@@ -2334,127 +2450,140 @@
       <c r="V10" s="12">
         <v>0</v>
       </c>
-      <c r="X10" s="8">
+      <c r="W10" s="5">
+        <v>0</v>
+      </c>
+      <c r="X10" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y10" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA10" s="8">
         <f t="shared" si="9"/>
         <v>45961</v>
       </c>
-      <c r="Y10" s="4">
+      <c r="AB10" s="4">
         <f t="shared" si="10"/>
         <v>270</v>
       </c>
-      <c r="Z10" s="4">
+      <c r="AC10" s="4">
         <f t="shared" si="26"/>
         <v>30</v>
       </c>
-      <c r="AA10" s="4">
+      <c r="AD10" s="4">
         <f t="shared" si="11"/>
         <v>284.74</v>
       </c>
-      <c r="AB10" s="4">
+      <c r="AE10" s="4">
         <f t="shared" si="12"/>
         <v>14.740000000000009</v>
       </c>
-      <c r="AC10" s="13">
+      <c r="AF10" s="13">
         <f t="shared" si="13"/>
         <v>5.4592592592592623E-2</v>
       </c>
-      <c r="AD10" s="4">
+      <c r="AG10" s="4">
         <f t="shared" si="27"/>
         <v>8.7300000000000182</v>
       </c>
-      <c r="AE10" s="10"/>
-      <c r="AF10" s="8">
+      <c r="AH10" s="10"/>
+      <c r="AI10" s="8">
         <f t="shared" si="14"/>
         <v>45961</v>
       </c>
-      <c r="AG10" s="4">
+      <c r="AJ10" s="4">
         <f t="shared" si="15"/>
         <v>1460</v>
       </c>
-      <c r="AH10" s="4">
+      <c r="AK10" s="4">
         <f t="shared" si="28"/>
         <v>20</v>
       </c>
-      <c r="AI10" s="4">
+      <c r="AL10" s="4">
         <f t="shared" si="16"/>
         <v>1570.02</v>
       </c>
-      <c r="AJ10" s="4">
+      <c r="AM10" s="4">
         <f t="shared" si="3"/>
         <v>110.01999999999998</v>
       </c>
-      <c r="AK10" s="13">
+      <c r="AN10" s="13">
         <f t="shared" si="4"/>
         <v>7.535616438356163E-2</v>
       </c>
-      <c r="AL10" s="4">
+      <c r="AO10" s="4">
         <f t="shared" si="29"/>
         <v>31.269999999999982</v>
       </c>
-      <c r="AM10" s="10"/>
-      <c r="AN10" s="8">
+      <c r="AP10" s="10"/>
+      <c r="AQ10" s="8">
         <f t="shared" si="17"/>
         <v>45961</v>
       </c>
-      <c r="AO10" s="4">
+      <c r="AR10" s="4">
         <f t="shared" si="18"/>
         <v>1730</v>
       </c>
-      <c r="AP10" s="4">
+      <c r="AS10" s="4">
         <f t="shared" si="30"/>
         <v>50</v>
       </c>
-      <c r="AQ10" s="4">
+      <c r="AT10" s="4">
         <f t="shared" si="19"/>
         <v>1854.76</v>
       </c>
-      <c r="AR10" s="4">
+      <c r="AU10" s="4">
         <f t="shared" si="5"/>
         <v>124.75999999999999</v>
       </c>
-      <c r="AS10" s="13">
+      <c r="AV10" s="13">
         <f t="shared" si="6"/>
         <v>7.2115606936416179E-2</v>
       </c>
-      <c r="AT10" s="4">
+      <c r="AW10" s="4">
         <f t="shared" si="31"/>
         <v>40</v>
       </c>
-      <c r="AV10" s="8">
+      <c r="AY10" s="8">
         <f t="shared" si="7"/>
         <v>45961</v>
       </c>
-      <c r="AW10" s="4">
+      <c r="AZ10" s="4">
         <f t="shared" si="20"/>
         <v>8.7300000000000182</v>
       </c>
-      <c r="AX10" s="4">
+      <c r="BA10" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="AY10" s="4">
+      <c r="BB10" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="AZ10" s="4">
+      <c r="BC10" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="BA10" s="4">
+      <c r="BD10" s="4">
         <f t="shared" si="24"/>
         <v>29.270000000000039</v>
       </c>
-      <c r="BB10" s="4">
+      <c r="BE10" s="4">
         <f t="shared" si="25"/>
         <v>2</v>
       </c>
-      <c r="BC10" s="4">
+      <c r="BF10" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
-      <c r="BD10" s="1"/>
+      <c r="BG10" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="BH10" s="1"/>
     </row>
-    <row r="11" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>45991</v>
       </c>
@@ -2494,7 +2623,7 @@
         <v>525</v>
       </c>
       <c r="M11" s="12">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v>0.05</v>
       </c>
       <c r="N11" s="5">
@@ -2504,7 +2633,7 @@
         <v>456.14</v>
       </c>
       <c r="P11" s="12">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v>8.6047619047619012E-2</v>
       </c>
       <c r="Q11" s="5">
@@ -2514,7 +2643,7 @@
         <v>634</v>
       </c>
       <c r="S11" s="12">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>3.9344262295081971E-2</v>
       </c>
       <c r="T11" s="5">
@@ -2526,127 +2655,140 @@
       <c r="V11" s="12">
         <v>0</v>
       </c>
-      <c r="X11" s="8">
+      <c r="W11" s="5">
+        <v>0</v>
+      </c>
+      <c r="X11" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y11" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA11" s="8">
         <f t="shared" si="9"/>
         <v>45991</v>
       </c>
-      <c r="Y11" s="4">
+      <c r="AB11" s="4">
         <f t="shared" si="10"/>
         <v>300</v>
       </c>
-      <c r="Z11" s="4">
+      <c r="AC11" s="4">
         <f t="shared" si="26"/>
         <v>30</v>
       </c>
-      <c r="AA11" s="4">
+      <c r="AD11" s="4">
         <f t="shared" si="11"/>
         <v>313.11</v>
       </c>
-      <c r="AB11" s="4">
+      <c r="AE11" s="4">
         <f t="shared" si="12"/>
         <v>13.110000000000014</v>
       </c>
-      <c r="AC11" s="13">
+      <c r="AF11" s="13">
         <f t="shared" si="13"/>
         <v>4.3700000000000044E-2</v>
       </c>
-      <c r="AD11" s="4">
+      <c r="AG11" s="4">
         <f t="shared" si="27"/>
         <v>-1.6299999999999955</v>
       </c>
-      <c r="AE11" s="10"/>
-      <c r="AF11" s="8">
+      <c r="AH11" s="10"/>
+      <c r="AI11" s="8">
         <f t="shared" si="14"/>
         <v>45991</v>
       </c>
-      <c r="AG11" s="4">
+      <c r="AJ11" s="4">
         <f t="shared" si="15"/>
         <v>1560</v>
       </c>
-      <c r="AH11" s="4">
+      <c r="AK11" s="4">
         <f t="shared" si="28"/>
         <v>100</v>
       </c>
-      <c r="AI11" s="4">
+      <c r="AL11" s="4">
         <f t="shared" si="16"/>
         <v>1700.19</v>
       </c>
-      <c r="AJ11" s="4">
+      <c r="AM11" s="4">
         <f t="shared" si="3"/>
         <v>140.19000000000005</v>
       </c>
-      <c r="AK11" s="13">
+      <c r="AN11" s="13">
         <f t="shared" si="4"/>
         <v>8.9865384615384653E-2</v>
       </c>
-      <c r="AL11" s="4">
+      <c r="AO11" s="4">
         <f t="shared" si="29"/>
         <v>30.170000000000073</v>
       </c>
-      <c r="AM11" s="10"/>
-      <c r="AN11" s="8">
+      <c r="AP11" s="10"/>
+      <c r="AQ11" s="8">
         <f t="shared" si="17"/>
         <v>45991</v>
       </c>
-      <c r="AO11" s="4">
+      <c r="AR11" s="4">
         <f t="shared" si="18"/>
         <v>1860</v>
       </c>
-      <c r="AP11" s="4">
+      <c r="AS11" s="4">
         <f t="shared" si="30"/>
         <v>130</v>
       </c>
-      <c r="AQ11" s="4">
+      <c r="AT11" s="4">
         <f t="shared" si="19"/>
         <v>2013.3000000000002</v>
       </c>
-      <c r="AR11" s="4">
+      <c r="AU11" s="4">
         <f t="shared" si="5"/>
         <v>153.30000000000018</v>
       </c>
-      <c r="AS11" s="13">
+      <c r="AV11" s="13">
         <f t="shared" si="6"/>
         <v>8.2419354838709769E-2</v>
       </c>
-      <c r="AT11" s="4">
+      <c r="AW11" s="4">
         <f t="shared" si="31"/>
         <v>28.540000000000191</v>
       </c>
-      <c r="AV11" s="8">
+      <c r="AY11" s="8">
         <f t="shared" si="7"/>
         <v>45991</v>
       </c>
-      <c r="AW11" s="4">
+      <c r="AZ11" s="4">
         <f t="shared" si="20"/>
         <v>-1.6299999999999955</v>
       </c>
-      <c r="AX11" s="4">
+      <c r="BA11" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="AY11" s="4">
+      <c r="BB11" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="AZ11" s="4">
+      <c r="BC11" s="4">
         <f t="shared" si="23"/>
         <v>25</v>
       </c>
-      <c r="BA11" s="4">
+      <c r="BD11" s="4">
         <f t="shared" si="24"/>
         <v>5.1699999999999591</v>
       </c>
-      <c r="BB11" s="4">
+      <c r="BE11" s="4">
         <f t="shared" si="25"/>
         <v>0</v>
       </c>
-      <c r="BC11" s="4">
+      <c r="BF11" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
-      <c r="BD11" s="1"/>
+      <c r="BG11" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="BH11" s="1"/>
     </row>
-    <row r="12" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
         <v>46022</v>
       </c>
@@ -2676,7 +2818,7 @@
         <v>85.1</v>
       </c>
       <c r="J12" s="12">
-        <f t="shared" ref="J12" si="36">(I12-H12)/H12</f>
+        <f t="shared" ref="J12" si="37">(I12-H12)/H12</f>
         <v>1.8366666666666664</v>
       </c>
       <c r="K12" s="19">
@@ -2686,7 +2828,7 @@
         <v>537.22</v>
       </c>
       <c r="M12" s="12">
-        <f t="shared" ref="M12" si="37">(L12-K12)/K12</f>
+        <f t="shared" ref="M12" si="38">(L12-K12)/K12</f>
         <v>7.4440000000000048E-2</v>
       </c>
       <c r="N12" s="5">
@@ -2696,7 +2838,7 @@
         <v>460.39</v>
       </c>
       <c r="P12" s="12">
-        <f t="shared" ref="P12" si="38">(O12-N12)/N12</f>
+        <f t="shared" ref="P12" si="39">(O12-N12)/N12</f>
         <v>9.6166666666666636E-2</v>
       </c>
       <c r="Q12" s="5">
@@ -2706,7 +2848,7 @@
         <v>634</v>
       </c>
       <c r="S12" s="12">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v>3.9344262295081971E-2</v>
       </c>
       <c r="T12" s="5">
@@ -2718,127 +2860,140 @@
       <c r="V12" s="12">
         <v>0</v>
       </c>
-      <c r="X12" s="8">
+      <c r="W12" s="5">
+        <v>0</v>
+      </c>
+      <c r="X12" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y12" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="8">
         <f t="shared" si="9"/>
         <v>46022</v>
       </c>
-      <c r="Y12" s="4">
+      <c r="AB12" s="4">
         <f t="shared" si="10"/>
         <v>300</v>
       </c>
-      <c r="Z12" s="4">
+      <c r="AC12" s="4">
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-      <c r="AA12" s="4">
+      <c r="AD12" s="4">
         <f t="shared" si="11"/>
         <v>317.85000000000002</v>
       </c>
-      <c r="AB12" s="4">
+      <c r="AE12" s="4">
         <f t="shared" si="12"/>
         <v>17.850000000000023</v>
       </c>
-      <c r="AC12" s="13">
+      <c r="AF12" s="13">
         <f t="shared" si="13"/>
         <v>5.9500000000000074E-2</v>
       </c>
-      <c r="AD12" s="4">
+      <c r="AG12" s="4">
         <f t="shared" si="27"/>
         <v>4.7400000000000091</v>
       </c>
-      <c r="AE12" s="10"/>
-      <c r="AF12" s="8">
+      <c r="AH12" s="10"/>
+      <c r="AI12" s="8">
         <f t="shared" si="14"/>
         <v>46022</v>
       </c>
-      <c r="AG12" s="4">
+      <c r="AJ12" s="4">
         <f t="shared" si="15"/>
         <v>1560</v>
       </c>
-      <c r="AH12" s="4">
+      <c r="AK12" s="4">
         <f t="shared" si="28"/>
         <v>0</v>
       </c>
-      <c r="AI12" s="4">
+      <c r="AL12" s="4">
         <f t="shared" si="16"/>
         <v>1716.71</v>
       </c>
-      <c r="AJ12" s="4">
+      <c r="AM12" s="4">
         <f t="shared" si="3"/>
         <v>156.71000000000004</v>
       </c>
-      <c r="AK12" s="13">
+      <c r="AN12" s="13">
         <f t="shared" si="4"/>
         <v>0.10045512820512822</v>
       </c>
-      <c r="AL12" s="4">
+      <c r="AO12" s="4">
         <f t="shared" si="29"/>
         <v>16.519999999999982</v>
       </c>
-      <c r="AM12" s="10"/>
-      <c r="AN12" s="8">
+      <c r="AP12" s="10"/>
+      <c r="AQ12" s="8">
         <f t="shared" si="17"/>
         <v>46022</v>
       </c>
-      <c r="AO12" s="4">
+      <c r="AR12" s="4">
         <f t="shared" si="18"/>
         <v>1860</v>
       </c>
-      <c r="AP12" s="4">
+      <c r="AS12" s="4">
         <f t="shared" si="30"/>
         <v>0</v>
       </c>
-      <c r="AQ12" s="4">
+      <c r="AT12" s="4">
         <f t="shared" si="19"/>
         <v>2034.56</v>
       </c>
-      <c r="AR12" s="4">
+      <c r="AU12" s="4">
         <f t="shared" si="5"/>
         <v>174.55999999999995</v>
       </c>
-      <c r="AS12" s="13">
+      <c r="AV12" s="13">
         <f t="shared" si="6"/>
         <v>9.3849462365591371E-2</v>
       </c>
-      <c r="AT12" s="4">
+      <c r="AW12" s="4">
         <f t="shared" si="31"/>
         <v>21.259999999999764</v>
       </c>
-      <c r="AV12" s="8">
+      <c r="AY12" s="8">
         <f t="shared" si="7"/>
         <v>46022</v>
       </c>
-      <c r="AW12" s="4">
+      <c r="AZ12" s="4">
         <f t="shared" si="20"/>
         <v>4.7400000000000091</v>
       </c>
-      <c r="AX12" s="4">
+      <c r="BA12" s="4">
         <f t="shared" si="21"/>
         <v>0</v>
       </c>
-      <c r="AY12" s="4">
+      <c r="BB12" s="4">
         <f t="shared" si="22"/>
         <v>4.9999999999997158E-2</v>
       </c>
-      <c r="AZ12" s="4">
+      <c r="BC12" s="4">
         <f t="shared" si="23"/>
         <v>12.220000000000027</v>
       </c>
-      <c r="BA12" s="4">
+      <c r="BD12" s="4">
         <f t="shared" si="24"/>
         <v>4.25</v>
       </c>
-      <c r="BB12" s="4">
+      <c r="BE12" s="4">
         <f t="shared" si="25"/>
         <v>0</v>
       </c>
-      <c r="BC12" s="4">
+      <c r="BF12" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
-      <c r="BD12" s="1"/>
+      <c r="BG12" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
+      <c r="BH12" s="1"/>
     </row>
-    <row r="13" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
         <v>46053</v>
       </c>
@@ -2849,7 +3004,7 @@
         <v>386.39</v>
       </c>
       <c r="D13" s="11">
-        <f t="shared" ref="D13" si="39">(C13-B13)/B13</f>
+        <f t="shared" ref="D13" si="40">(C13-B13)/B13</f>
         <v>7.3305555555555513E-2</v>
       </c>
       <c r="E13" s="5">
@@ -2859,7 +3014,7 @@
         <v>99.06</v>
       </c>
       <c r="G13" s="11">
-        <f t="shared" ref="G13" si="40">(F13-E13)/E13</f>
+        <f t="shared" ref="G13" si="41">(F13-E13)/E13</f>
         <v>-9.3999999999999778E-3</v>
       </c>
       <c r="H13" s="5">
@@ -2869,7 +3024,7 @@
         <v>85.1</v>
       </c>
       <c r="J13" s="12">
-        <f t="shared" ref="J13" si="41">(I13-H13)/H13</f>
+        <f t="shared" ref="J13" si="42">(I13-H13)/H13</f>
         <v>1.8366666666666664</v>
       </c>
       <c r="K13" s="19">
@@ -2879,7 +3034,7 @@
         <v>537.22</v>
       </c>
       <c r="M13" s="12">
-        <f t="shared" ref="M13" si="42">(L13-K13)/K13</f>
+        <f t="shared" ref="M13" si="43">(L13-K13)/K13</f>
         <v>7.4440000000000048E-2</v>
       </c>
       <c r="N13" s="5">
@@ -2889,7 +3044,7 @@
         <v>464.76</v>
       </c>
       <c r="P13" s="12">
-        <f t="shared" ref="P13" si="43">(O13-N13)/N13</f>
+        <f t="shared" ref="P13" si="44">(O13-N13)/N13</f>
         <v>0.10657142857142855</v>
       </c>
       <c r="Q13" s="5">
@@ -2899,7 +3054,7 @@
         <v>634</v>
       </c>
       <c r="S13" s="12">
-        <f t="shared" ref="S13" si="44">(R13-Q13)/Q13</f>
+        <f t="shared" ref="S13" si="45">(R13-Q13)/Q13</f>
         <v>3.9344262295081971E-2</v>
       </c>
       <c r="T13" s="5">
@@ -2911,126 +3066,139 @@
       <c r="V13" s="12">
         <v>0</v>
       </c>
-      <c r="X13" s="8">
+      <c r="W13" s="5">
+        <v>0</v>
+      </c>
+      <c r="X13" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="8">
         <f t="shared" si="9"/>
         <v>46053</v>
       </c>
-      <c r="Y13" s="4">
+      <c r="AB13" s="4">
         <f t="shared" si="10"/>
         <v>460</v>
       </c>
-      <c r="Z13" s="4">
+      <c r="AC13" s="4">
         <f t="shared" si="26"/>
         <v>160</v>
       </c>
-      <c r="AA13" s="4">
+      <c r="AD13" s="4">
         <f t="shared" si="11"/>
         <v>485.45</v>
       </c>
-      <c r="AB13" s="4">
+      <c r="AE13" s="4">
         <f t="shared" si="12"/>
         <v>25.449999999999989</v>
       </c>
-      <c r="AC13" s="13">
+      <c r="AF13" s="13">
         <f t="shared" si="13"/>
         <v>5.5326086956521713E-2</v>
       </c>
-      <c r="AD13" s="4">
+      <c r="AG13" s="4">
         <f t="shared" si="27"/>
         <v>7.5999999999999659</v>
       </c>
-      <c r="AE13" s="10"/>
-      <c r="AF13" s="8">
+      <c r="AH13" s="10"/>
+      <c r="AI13" s="8">
         <f t="shared" si="14"/>
         <v>46053</v>
       </c>
-      <c r="AG13" s="4">
+      <c r="AJ13" s="4">
         <f t="shared" si="15"/>
         <v>1560</v>
       </c>
-      <c r="AH13" s="4">
+      <c r="AK13" s="4">
         <f t="shared" si="28"/>
         <v>0</v>
       </c>
-      <c r="AI13" s="4">
+      <c r="AL13" s="4">
         <f t="shared" si="16"/>
         <v>1721.08</v>
       </c>
-      <c r="AJ13" s="4">
+      <c r="AM13" s="4">
         <f t="shared" si="3"/>
         <v>161.07999999999993</v>
       </c>
-      <c r="AK13" s="13">
+      <c r="AN13" s="13">
         <f t="shared" si="4"/>
         <v>0.10325641025641021</v>
       </c>
-      <c r="AL13" s="4">
+      <c r="AO13" s="4">
         <f t="shared" si="29"/>
         <v>4.3699999999998909</v>
       </c>
-      <c r="AM13" s="10"/>
-      <c r="AN13" s="8">
+      <c r="AP13" s="10"/>
+      <c r="AQ13" s="8">
         <f t="shared" si="17"/>
         <v>46053</v>
       </c>
-      <c r="AO13" s="4">
+      <c r="AR13" s="4">
         <f t="shared" si="18"/>
         <v>2020</v>
       </c>
-      <c r="AP13" s="4">
+      <c r="AS13" s="4">
         <f t="shared" si="30"/>
         <v>160</v>
       </c>
-      <c r="AQ13" s="4">
+      <c r="AT13" s="4">
         <f t="shared" si="19"/>
         <v>2206.5299999999997</v>
       </c>
-      <c r="AR13" s="4">
+      <c r="AU13" s="4">
         <f t="shared" si="5"/>
         <v>186.52999999999975</v>
       </c>
-      <c r="AS13" s="13">
+      <c r="AV13" s="13">
         <f t="shared" si="6"/>
         <v>9.2341584158415715E-2</v>
       </c>
-      <c r="AT13" s="4">
+      <c r="AW13" s="4">
         <f t="shared" si="31"/>
         <v>11.9699999999998</v>
       </c>
-      <c r="AV13" s="8">
+      <c r="AY13" s="8">
         <f t="shared" si="7"/>
         <v>46053</v>
       </c>
-      <c r="AW13" s="4">
+      <c r="AZ13" s="4">
         <f t="shared" si="20"/>
         <v>8.5399999999999636</v>
       </c>
-      <c r="AX13" s="4">
+      <c r="BA13" s="4">
         <f t="shared" si="21"/>
         <v>-0.93999999999999773</v>
       </c>
-      <c r="AY13" s="4">
+      <c r="BB13" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="AZ13" s="4">
+      <c r="BC13" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="BA13" s="4">
+      <c r="BD13" s="4">
         <f t="shared" si="24"/>
         <v>4.3700000000000045</v>
       </c>
-      <c r="BB13" s="4">
+      <c r="BE13" s="4">
         <f t="shared" si="25"/>
         <v>0</v>
       </c>
-      <c r="BC13" s="4">
+      <c r="BF13" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
+      <c r="BG13" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="14" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
         <v>46081</v>
       </c>
@@ -3041,7 +3209,7 @@
         <v>421.42</v>
       </c>
       <c r="D14" s="11">
-        <f t="shared" ref="D14" si="45">(C14-B14)/B14</f>
+        <f t="shared" ref="D14" si="46">(C14-B14)/B14</f>
         <v>8.056410256410261E-2</v>
       </c>
       <c r="E14" s="5">
@@ -3051,7 +3219,7 @@
         <v>201.06</v>
       </c>
       <c r="G14" s="11">
-        <f t="shared" ref="G14" si="46">(F14-E14)/E14</f>
+        <f t="shared" ref="G14" si="47">(F14-E14)/E14</f>
         <v>5.3000000000000113E-3</v>
       </c>
       <c r="H14" s="5">
@@ -3061,7 +3229,7 @@
         <v>85.1</v>
       </c>
       <c r="J14" s="12">
-        <f t="shared" ref="J14" si="47">(I14-H14)/H14</f>
+        <f t="shared" ref="J14" si="48">(I14-H14)/H14</f>
         <v>1.8366666666666664</v>
       </c>
       <c r="K14" s="19">
@@ -3071,7 +3239,7 @@
         <v>537.22</v>
       </c>
       <c r="M14" s="12">
-        <f t="shared" ref="M14" si="48">(L14-K14)/K14</f>
+        <f t="shared" ref="M14" si="49">(L14-K14)/K14</f>
         <v>7.4440000000000048E-2</v>
       </c>
       <c r="N14" s="5">
@@ -3081,7 +3249,7 @@
         <v>469.11</v>
       </c>
       <c r="P14" s="12">
-        <f t="shared" ref="P14" si="49">(O14-N14)/N14</f>
+        <f t="shared" ref="P14" si="50">(O14-N14)/N14</f>
         <v>0.11692857142857147</v>
       </c>
       <c r="Q14" s="5">
@@ -3091,7 +3259,7 @@
         <v>644.72</v>
       </c>
       <c r="S14" s="12">
-        <f t="shared" ref="S14" si="50">(R14-Q14)/Q14</f>
+        <f t="shared" ref="S14" si="51">(R14-Q14)/Q14</f>
         <v>5.6918032786885293E-2</v>
       </c>
       <c r="T14" s="5">
@@ -3103,126 +3271,139 @@
       <c r="V14" s="12">
         <v>0</v>
       </c>
-      <c r="X14" s="8">
+      <c r="W14" s="5">
+        <v>0</v>
+      </c>
+      <c r="X14" s="4">
+        <v>0</v>
+      </c>
+      <c r="Y14" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA14" s="8">
         <f t="shared" si="9"/>
         <v>46081</v>
       </c>
-      <c r="Y14" s="4">
+      <c r="AB14" s="4">
         <f t="shared" si="10"/>
         <v>590</v>
       </c>
-      <c r="Z14" s="4">
+      <c r="AC14" s="4">
         <f t="shared" si="26"/>
         <v>130</v>
       </c>
-      <c r="AA14" s="4">
+      <c r="AD14" s="4">
         <f t="shared" si="11"/>
         <v>622.48</v>
       </c>
-      <c r="AB14" s="4">
+      <c r="AE14" s="4">
         <f t="shared" si="12"/>
         <v>32.480000000000018</v>
       </c>
-      <c r="AC14" s="13">
+      <c r="AF14" s="13">
         <f t="shared" si="13"/>
         <v>5.5050847457627151E-2</v>
       </c>
-      <c r="AD14" s="4">
+      <c r="AG14" s="4">
         <f t="shared" si="27"/>
         <v>7.0300000000000296</v>
       </c>
-      <c r="AE14" s="10"/>
-      <c r="AF14" s="8">
+      <c r="AH14" s="10"/>
+      <c r="AI14" s="8">
         <f t="shared" si="14"/>
         <v>46081</v>
       </c>
-      <c r="AG14" s="4">
+      <c r="AJ14" s="4">
         <f t="shared" si="15"/>
         <v>1560</v>
       </c>
-      <c r="AH14" s="4">
+      <c r="AK14" s="4">
         <f t="shared" si="28"/>
         <v>0</v>
       </c>
-      <c r="AI14" s="4">
+      <c r="AL14" s="4">
         <f t="shared" si="16"/>
         <v>1736.15</v>
       </c>
-      <c r="AJ14" s="4">
+      <c r="AM14" s="4">
         <f t="shared" si="3"/>
         <v>176.15000000000009</v>
       </c>
-      <c r="AK14" s="13">
+      <c r="AN14" s="13">
         <f t="shared" si="4"/>
         <v>0.11291666666666672</v>
       </c>
-      <c r="AL14" s="4">
+      <c r="AO14" s="4">
         <f t="shared" si="29"/>
         <v>15.070000000000164</v>
       </c>
-      <c r="AM14" s="10"/>
-      <c r="AN14" s="8">
+      <c r="AP14" s="10"/>
+      <c r="AQ14" s="8">
         <f t="shared" si="17"/>
         <v>46081</v>
       </c>
-      <c r="AO14" s="4">
+      <c r="AR14" s="4">
         <f t="shared" si="18"/>
         <v>2150</v>
       </c>
-      <c r="AP14" s="4">
+      <c r="AS14" s="4">
         <f t="shared" si="30"/>
         <v>130</v>
       </c>
-      <c r="AQ14" s="4">
+      <c r="AT14" s="4">
         <f t="shared" si="19"/>
         <v>2358.63</v>
       </c>
-      <c r="AR14" s="4">
+      <c r="AU14" s="4">
         <f t="shared" si="5"/>
         <v>208.63000000000011</v>
       </c>
-      <c r="AS14" s="13">
+      <c r="AV14" s="13">
         <f t="shared" si="6"/>
         <v>9.7037209302325636E-2</v>
       </c>
-      <c r="AT14" s="4">
+      <c r="AW14" s="4">
         <f t="shared" si="31"/>
         <v>22.100000000000364</v>
       </c>
-      <c r="AV14" s="8">
+      <c r="AY14" s="8">
         <f t="shared" si="7"/>
         <v>46081</v>
       </c>
-      <c r="AW14" s="4">
+      <c r="AZ14" s="4">
         <f t="shared" si="20"/>
         <v>5.0300000000000296</v>
       </c>
-      <c r="AX14" s="4">
+      <c r="BA14" s="4">
         <f t="shared" si="21"/>
         <v>2</v>
       </c>
-      <c r="AY14" s="4">
+      <c r="BB14" s="4">
         <f t="shared" si="22"/>
         <v>0</v>
       </c>
-      <c r="AZ14" s="4">
+      <c r="BC14" s="4">
         <f t="shared" si="23"/>
         <v>0</v>
       </c>
-      <c r="BA14" s="4">
+      <c r="BD14" s="4">
         <f t="shared" si="24"/>
         <v>4.3500000000000227</v>
       </c>
-      <c r="BB14" s="4">
+      <c r="BE14" s="4">
         <f t="shared" si="25"/>
         <v>10.720000000000027</v>
       </c>
-      <c r="BC14" s="4">
+      <c r="BF14" s="4">
         <f t="shared" si="32"/>
         <v>0</v>
       </c>
+      <c r="BG14" s="4">
+        <f t="shared" si="33"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>46112</v>
       </c>
@@ -3233,7 +3414,7 @@
         <v>418.68</v>
       </c>
       <c r="D15" s="11">
-        <f t="shared" ref="D15" si="51">(C15-B15)/B15</f>
+        <f t="shared" ref="D15" si="52">(C15-B15)/B15</f>
         <v>-3.1428571428571265E-3</v>
       </c>
       <c r="E15" s="5">
@@ -3243,7 +3424,7 @@
         <v>292.23</v>
       </c>
       <c r="G15" s="11">
-        <f t="shared" ref="G15" si="52">(F15-E15)/E15</f>
+        <f t="shared" ref="G15" si="53">(F15-E15)/E15</f>
         <v>-2.589999999999994E-2</v>
       </c>
       <c r="H15" s="5">
@@ -3253,7 +3434,7 @@
         <v>85.1</v>
       </c>
       <c r="J15" s="12">
-        <f t="shared" ref="J15" si="53">(I15-H15)/H15</f>
+        <f t="shared" ref="J15" si="54">(I15-H15)/H15</f>
         <v>1.8366666666666664</v>
       </c>
       <c r="K15" s="19">
@@ -3263,7 +3444,7 @@
         <v>544.55999999999995</v>
       </c>
       <c r="M15" s="12">
-        <f t="shared" ref="M15" si="54">(L15-K15)/K15</f>
+        <f t="shared" ref="M15" si="55">(L15-K15)/K15</f>
         <v>8.9119999999999894E-2</v>
       </c>
       <c r="N15" s="5">
@@ -3273,7 +3454,7 @@
         <v>677.43</v>
       </c>
       <c r="P15" s="12">
-        <f t="shared" ref="P15" si="55">(O15-N15)/N15</f>
+        <f t="shared" ref="P15" si="56">(O15-N15)/N15</f>
         <v>9.2629032258064431E-2</v>
       </c>
       <c r="Q15" s="5">
@@ -3283,7 +3464,7 @@
         <v>654.46</v>
       </c>
       <c r="S15" s="12">
-        <f t="shared" ref="S15" si="56">(R15-Q15)/Q15</f>
+        <f t="shared" ref="S15" si="57">(R15-Q15)/Q15</f>
         <v>7.2885245901639403E-2</v>
       </c>
       <c r="T15" s="5">
@@ -3295,126 +3476,139 @@
       <c r="V15" s="12">
         <v>0</v>
       </c>
-      <c r="X15" s="8">
-        <f t="shared" ref="X15" si="57">A15</f>
+      <c r="W15" s="5">
+        <v>0</v>
+      </c>
+      <c r="X15" s="4">
+        <v>10</v>
+      </c>
+      <c r="Y15" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA15" s="8">
+        <f t="shared" ref="AA15" si="58">A15</f>
         <v>46112</v>
       </c>
-      <c r="Y15" s="4">
+      <c r="AB15" s="4">
         <f t="shared" si="10"/>
         <v>720</v>
       </c>
-      <c r="Z15" s="4">
+      <c r="AC15" s="4">
         <f t="shared" si="26"/>
         <v>130</v>
       </c>
-      <c r="AA15" s="4">
+      <c r="AD15" s="4">
         <f t="shared" si="11"/>
         <v>710.91000000000008</v>
       </c>
-      <c r="AB15" s="4">
-        <f t="shared" ref="AB15" si="58">AA15-Y15</f>
+      <c r="AE15" s="4">
+        <f t="shared" ref="AE15" si="59">AD15-AB15</f>
         <v>-9.0899999999999181</v>
       </c>
-      <c r="AC15" s="13">
-        <f t="shared" ref="AC15" si="59">AB15/Y15</f>
+      <c r="AF15" s="13">
+        <f t="shared" ref="AF15" si="60">AE15/AB15</f>
         <v>-1.2624999999999886E-2</v>
       </c>
-      <c r="AD15" s="4">
-        <f t="shared" ref="AD15" si="60">AB15-AB14</f>
+      <c r="AG15" s="4">
+        <f t="shared" ref="AG15" si="61">AE15-AE14</f>
         <v>-41.569999999999936</v>
       </c>
-      <c r="AE15" s="10"/>
-      <c r="AF15" s="8">
+      <c r="AH15" s="10"/>
+      <c r="AI15" s="8">
         <f t="shared" si="14"/>
         <v>46112</v>
       </c>
-      <c r="AG15" s="4">
+      <c r="AJ15" s="4">
         <f t="shared" si="15"/>
         <v>1760</v>
       </c>
-      <c r="AH15" s="4">
+      <c r="AK15" s="4">
         <f t="shared" si="28"/>
         <v>200</v>
       </c>
-      <c r="AI15" s="4">
+      <c r="AL15" s="4">
         <f t="shared" si="16"/>
-        <v>1971.55</v>
-      </c>
-      <c r="AJ15" s="4">
+        <v>1981.55</v>
+      </c>
+      <c r="AM15" s="4">
         <f t="shared" si="3"/>
-        <v>211.54999999999995</v>
-      </c>
-      <c r="AK15" s="13">
+        <v>221.54999999999995</v>
+      </c>
+      <c r="AN15" s="13">
         <f t="shared" si="4"/>
-        <v>0.1201988636363636</v>
-      </c>
-      <c r="AL15" s="4">
+        <v>0.12588068181818179</v>
+      </c>
+      <c r="AO15" s="4">
         <f t="shared" si="29"/>
-        <v>35.399999999999864</v>
-      </c>
-      <c r="AM15" s="10"/>
-      <c r="AN15" s="8">
+        <v>45.399999999999864</v>
+      </c>
+      <c r="AP15" s="10"/>
+      <c r="AQ15" s="8">
         <f t="shared" si="17"/>
         <v>46112</v>
       </c>
-      <c r="AO15" s="4">
+      <c r="AR15" s="4">
         <f t="shared" si="18"/>
         <v>2480</v>
       </c>
-      <c r="AP15" s="4">
+      <c r="AS15" s="4">
         <f t="shared" si="30"/>
         <v>330</v>
       </c>
-      <c r="AQ15" s="4">
+      <c r="AT15" s="4">
         <f t="shared" si="19"/>
-        <v>2682.46</v>
-      </c>
-      <c r="AR15" s="4">
+        <v>2692.46</v>
+      </c>
+      <c r="AU15" s="4">
         <f t="shared" si="5"/>
-        <v>202.46000000000004</v>
-      </c>
-      <c r="AS15" s="13">
+        <v>212.46000000000004</v>
+      </c>
+      <c r="AV15" s="13">
         <f t="shared" si="6"/>
-        <v>8.1637096774193563E-2</v>
-      </c>
-      <c r="AT15" s="4">
+        <v>8.5669354838709688E-2</v>
+      </c>
+      <c r="AW15" s="4">
         <f t="shared" si="31"/>
-        <v>-6.1700000000000728</v>
-      </c>
-      <c r="AV15" s="8">
-        <f t="shared" ref="AV15" si="61">A15</f>
+        <v>3.8299999999999272</v>
+      </c>
+      <c r="AY15" s="8">
+        <f t="shared" ref="AY15" si="62">A15</f>
         <v>46112</v>
       </c>
-      <c r="AW15" s="4">
-        <f t="shared" ref="AW15" si="62">(C15-B15)-(C14-B14)</f>
+      <c r="AZ15" s="4">
+        <f t="shared" ref="AZ15" si="63">(C15-B15)-(C14-B14)</f>
         <v>-32.740000000000009</v>
       </c>
-      <c r="AX15" s="4">
-        <f t="shared" ref="AX15" si="63">(F15-E15)-(F14-E14)</f>
+      <c r="BA15" s="4">
+        <f t="shared" ref="BA15" si="64">(F15-E15)-(F14-E14)</f>
         <v>-8.8299999999999841</v>
       </c>
-      <c r="AY15" s="4">
-        <f t="shared" ref="AY15" si="64">(I15-H15)-(I14-H14)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ15" s="4">
-        <f t="shared" ref="AZ15" si="65">(L15-K15)-(L14-K14)</f>
+      <c r="BB15" s="4">
+        <f t="shared" ref="BB15" si="65">(I15-H15)-(I14-H14)</f>
+        <v>0</v>
+      </c>
+      <c r="BC15" s="4">
+        <f t="shared" ref="BC15" si="66">(L15-K15)-(L14-K14)</f>
         <v>7.3399999999999181</v>
       </c>
-      <c r="BA15" s="4">
-        <f t="shared" ref="BA15" si="66">(O15-N15)-(O14-N14)</f>
+      <c r="BD15" s="4">
+        <f t="shared" ref="BD15" si="67">(O15-N15)-(O14-N14)</f>
         <v>8.3199999999999363</v>
       </c>
-      <c r="BB15" s="4">
-        <f t="shared" ref="BB15" si="67">(R15-Q15)-(R14-Q14)</f>
+      <c r="BE15" s="4">
+        <f t="shared" ref="BE15" si="68">(R15-Q15)-(R14-Q14)</f>
         <v>9.7400000000000091</v>
       </c>
-      <c r="BC15" s="4">
+      <c r="BF15" s="4">
         <f t="shared" si="32"/>
         <v>10</v>
       </c>
+      <c r="BG15" s="4">
+        <f t="shared" si="33"/>
+        <v>10</v>
+      </c>
     </row>
-    <row r="16" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:60" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
         <v>46142</v>
       </c>
@@ -3425,7 +3619,7 @@
         <v>476.59</v>
       </c>
       <c r="D16" s="11">
-        <f t="shared" ref="D16" si="68">(C16-B16)/B16</f>
+        <f t="shared" ref="D16" si="69">(C16-B16)/B16</f>
         <v>5.9088888888888837E-2</v>
       </c>
       <c r="E16" s="5">
@@ -3435,7 +3629,7 @@
         <v>418.03</v>
       </c>
       <c r="G16" s="11">
-        <f t="shared" ref="G16" si="69">(F16-E16)/E16</f>
+        <f t="shared" ref="G16" si="70">(F16-E16)/E16</f>
         <v>4.5074999999999935E-2</v>
       </c>
       <c r="H16" s="5">
@@ -3445,7 +3639,7 @@
         <v>85.1</v>
       </c>
       <c r="J16" s="12">
-        <f t="shared" ref="J16" si="70">(I16-H16)/H16</f>
+        <f t="shared" ref="J16" si="71">(I16-H16)/H16</f>
         <v>1.8366666666666664</v>
       </c>
       <c r="K16" s="19">
@@ -3455,7 +3649,7 @@
         <v>549.24</v>
       </c>
       <c r="M16" s="12">
-        <f t="shared" ref="M16" si="71">(L16-K16)/K16</f>
+        <f t="shared" ref="M16" si="72">(L16-K16)/K16</f>
         <v>9.8480000000000012E-2</v>
       </c>
       <c r="N16" s="5">
@@ -3465,7 +3659,7 @@
         <v>679.75</v>
       </c>
       <c r="P16" s="12">
-        <f t="shared" ref="P16" si="72">(O16-N16)/N16</f>
+        <f t="shared" ref="P16" si="73">(O16-N16)/N16</f>
         <v>9.6370967741935487E-2</v>
       </c>
       <c r="Q16" s="5">
@@ -3475,7 +3669,7 @@
         <v>664.55</v>
       </c>
       <c r="S16" s="12">
-        <f t="shared" ref="S16" si="73">(R16-Q16)/Q16</f>
+        <f t="shared" ref="S16" si="74">(R16-Q16)/Q16</f>
         <v>8.9426229508196647E-2</v>
       </c>
       <c r="T16" s="5">
@@ -3488,126 +3682,139 @@
         <f>(U16-T16)/T16</f>
         <v>0.25250000000000006</v>
       </c>
-      <c r="X16" s="8">
-        <f t="shared" ref="X16" si="74">A16</f>
+      <c r="W16" s="5">
+        <v>0</v>
+      </c>
+      <c r="X16" s="4">
+        <v>10</v>
+      </c>
+      <c r="Y16" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA16" s="8">
+        <f t="shared" ref="AA16" si="75">A16</f>
         <v>46142</v>
       </c>
-      <c r="Y16" s="4">
+      <c r="AB16" s="4">
         <f t="shared" si="10"/>
         <v>850</v>
       </c>
-      <c r="Z16" s="4">
+      <c r="AC16" s="4">
         <f t="shared" si="26"/>
         <v>130</v>
       </c>
-      <c r="AA16" s="4">
+      <c r="AD16" s="4">
         <f t="shared" si="11"/>
         <v>894.61999999999989</v>
       </c>
-      <c r="AB16" s="4">
-        <f t="shared" ref="AB16" si="75">AA16-Y16</f>
+      <c r="AE16" s="4">
+        <f t="shared" ref="AE16" si="76">AD16-AB16</f>
         <v>44.619999999999891</v>
       </c>
-      <c r="AC16" s="13">
-        <f t="shared" ref="AC16" si="76">AB16/Y16</f>
+      <c r="AF16" s="13">
+        <f t="shared" ref="AF16" si="77">AE16/AB16</f>
         <v>5.2494117647058698E-2</v>
       </c>
-      <c r="AD16" s="4">
-        <f t="shared" ref="AD16" si="77">AB16-AB15</f>
+      <c r="AG16" s="4">
+        <f t="shared" ref="AG16" si="78">AE16-AE15</f>
         <v>53.709999999999809</v>
       </c>
-      <c r="AE16" s="10"/>
-      <c r="AF16" s="8">
+      <c r="AH16" s="10"/>
+      <c r="AI16" s="8">
         <f t="shared" si="14"/>
         <v>46142</v>
       </c>
-      <c r="AG16" s="4">
+      <c r="AJ16" s="4">
         <f t="shared" si="15"/>
         <v>1800</v>
       </c>
-      <c r="AH16" s="4">
+      <c r="AK16" s="4">
         <f t="shared" si="28"/>
         <v>40</v>
       </c>
-      <c r="AI16" s="4">
+      <c r="AL16" s="4">
         <f t="shared" si="16"/>
-        <v>2028.74</v>
-      </c>
-      <c r="AJ16" s="4">
+        <v>2038.74</v>
+      </c>
+      <c r="AM16" s="4">
         <f t="shared" si="3"/>
-        <v>228.74</v>
-      </c>
-      <c r="AK16" s="13">
+        <v>238.74</v>
+      </c>
+      <c r="AN16" s="13">
         <f t="shared" si="4"/>
-        <v>0.12707777777777779</v>
-      </c>
-      <c r="AL16" s="4">
+        <v>0.13263333333333333</v>
+      </c>
+      <c r="AO16" s="4">
         <f t="shared" si="29"/>
         <v>17.190000000000055</v>
       </c>
-      <c r="AM16" s="10"/>
-      <c r="AN16" s="8">
+      <c r="AP16" s="10"/>
+      <c r="AQ16" s="8">
         <f t="shared" si="17"/>
         <v>46142</v>
       </c>
-      <c r="AO16" s="4">
+      <c r="AR16" s="4">
         <f t="shared" si="18"/>
         <v>2650</v>
       </c>
-      <c r="AP16" s="4">
+      <c r="AS16" s="4">
         <f t="shared" si="30"/>
         <v>170</v>
       </c>
-      <c r="AQ16" s="4">
+      <c r="AT16" s="4">
         <f t="shared" si="19"/>
-        <v>2923.3599999999997</v>
-      </c>
-      <c r="AR16" s="4">
+        <v>2933.3599999999997</v>
+      </c>
+      <c r="AU16" s="4">
         <f t="shared" si="5"/>
-        <v>273.35999999999967</v>
-      </c>
-      <c r="AS16" s="13">
+        <v>283.35999999999967</v>
+      </c>
+      <c r="AV16" s="13">
         <f t="shared" si="6"/>
-        <v>0.10315471698113195</v>
-      </c>
-      <c r="AT16" s="4">
+        <v>0.10692830188679232</v>
+      </c>
+      <c r="AW16" s="4">
         <f t="shared" si="31"/>
         <v>70.899999999999636</v>
       </c>
-      <c r="AV16" s="8">
-        <f t="shared" ref="AV16" si="78">A16</f>
+      <c r="AY16" s="8">
+        <f t="shared" ref="AY16" si="79">A16</f>
         <v>46142</v>
       </c>
-      <c r="AW16" s="4">
-        <f t="shared" ref="AW16" si="79">(C16-B16)-(C15-B15)</f>
+      <c r="AZ16" s="4">
+        <f t="shared" ref="AZ16" si="80">(C16-B16)-(C15-B15)</f>
         <v>27.909999999999968</v>
       </c>
-      <c r="AX16" s="4">
-        <f t="shared" ref="AX16" si="80">(F16-E16)-(F15-E15)</f>
+      <c r="BA16" s="4">
+        <f t="shared" ref="BA16" si="81">(F16-E16)-(F15-E15)</f>
         <v>25.799999999999955</v>
       </c>
-      <c r="AY16" s="4">
-        <f t="shared" ref="AY16" si="81">(I16-H16)-(I15-H15)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ16" s="4">
-        <f t="shared" ref="AZ16" si="82">(L16-K16)-(L15-K15)</f>
+      <c r="BB16" s="4">
+        <f t="shared" ref="BB16" si="82">(I16-H16)-(I15-H15)</f>
+        <v>0</v>
+      </c>
+      <c r="BC16" s="4">
+        <f t="shared" ref="BC16" si="83">(L16-K16)-(L15-K15)</f>
         <v>4.6800000000000637</v>
       </c>
-      <c r="BA16" s="4">
-        <f t="shared" ref="BA16" si="83">(O16-N16)-(O15-N15)</f>
+      <c r="BD16" s="4">
+        <f t="shared" ref="BD16" si="84">(O16-N16)-(O15-N15)</f>
         <v>2.32000000000005</v>
       </c>
-      <c r="BB16" s="4">
-        <f t="shared" ref="BB16" si="84">(R16-Q16)-(R15-Q15)</f>
+      <c r="BE16" s="4">
+        <f t="shared" ref="BE16" si="85">(R16-Q16)-(R15-Q15)</f>
         <v>10.089999999999918</v>
       </c>
-      <c r="BC16" s="4">
-        <f t="shared" ref="BC16" si="85">(U16-T16)-(U15-T15)</f>
+      <c r="BF16" s="4">
+        <f t="shared" si="32"/>
         <v>0.10000000000000142</v>
       </c>
+      <c r="BG16" s="4">
+        <f t="shared" ref="BF16:BG16" si="86">(X16-W16)-(X15-W15)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>46173</v>
       </c>
@@ -3618,7 +3825,7 @@
         <v>527.07000000000005</v>
       </c>
       <c r="D17" s="11">
-        <f t="shared" ref="D17" si="86">(C17-B17)/B17</f>
+        <f t="shared" ref="D17" si="87">(C17-B17)/B17</f>
         <v>9.8062500000000108E-2</v>
       </c>
       <c r="E17" s="5">
@@ -3628,7 +3835,7 @@
         <v>544.42999999999995</v>
       </c>
       <c r="G17" s="11">
-        <f t="shared" ref="G17" si="87">(F17-E17)/E17</f>
+        <f t="shared" ref="G17" si="88">(F17-E17)/E17</f>
         <v>8.8859999999999897E-2</v>
       </c>
       <c r="H17" s="5">
@@ -3638,7 +3845,7 @@
         <v>85.35</v>
       </c>
       <c r="J17" s="12">
-        <f t="shared" ref="J17" si="88">(I17-H17)/H17</f>
+        <f t="shared" ref="J17" si="89">(I17-H17)/H17</f>
         <v>1.8449999999999998</v>
       </c>
       <c r="K17" s="19">
@@ -3648,7 +3855,7 @@
         <v>551.17999999999995</v>
       </c>
       <c r="M17" s="12">
-        <f t="shared" ref="M17" si="89">(L17-K17)/K17</f>
+        <f t="shared" ref="M17" si="90">(L17-K17)/K17</f>
         <v>6.9442558062826135E-2</v>
       </c>
       <c r="N17" s="5">
@@ -3658,7 +3865,7 @@
         <v>684.13</v>
       </c>
       <c r="P17" s="12">
-        <f t="shared" ref="P17" si="90">(O17-N17)/N17</f>
+        <f t="shared" ref="P17" si="91">(O17-N17)/N17</f>
         <v>0.10343548387096774</v>
       </c>
       <c r="Q17" s="5">
@@ -3668,7 +3875,7 @@
         <v>666.19</v>
       </c>
       <c r="S17" s="12">
-        <f t="shared" ref="S17" si="91">(R17-Q17)/Q17</f>
+        <f t="shared" ref="S17" si="92">(R17-Q17)/Q17</f>
         <v>9.2114754098360743E-2</v>
       </c>
       <c r="T17" s="5">
@@ -3681,126 +3888,139 @@
         <f>(U17-T17)/T17</f>
         <v>0.15</v>
       </c>
-      <c r="X17" s="8">
-        <f t="shared" ref="X17" si="92">A17</f>
+      <c r="W17" s="5">
+        <v>0</v>
+      </c>
+      <c r="X17" s="4">
+        <v>10</v>
+      </c>
+      <c r="Y17" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA17" s="8">
+        <f t="shared" ref="AA17" si="93">A17</f>
         <v>46173</v>
       </c>
-      <c r="Y17" s="4">
-        <f t="shared" ref="Y17" si="93">B17+E17</f>
+      <c r="AB17" s="4">
+        <f t="shared" ref="AB17" si="94">B17+E17</f>
         <v>980</v>
       </c>
-      <c r="Z17" s="4">
-        <f t="shared" ref="Z17" si="94">Y17-Y16</f>
+      <c r="AC17" s="4">
+        <f t="shared" ref="AC17" si="95">AB17-AB16</f>
         <v>130</v>
       </c>
-      <c r="AA17" s="4">
-        <f t="shared" ref="AA17" si="95">C17+F17</f>
+      <c r="AD17" s="4">
+        <f t="shared" ref="AD17" si="96">C17+F17</f>
         <v>1071.5</v>
       </c>
-      <c r="AB17" s="4">
-        <f t="shared" ref="AB17" si="96">AA17-Y17</f>
+      <c r="AE17" s="4">
+        <f t="shared" ref="AE17" si="97">AD17-AB17</f>
         <v>91.5</v>
       </c>
-      <c r="AC17" s="13">
-        <f t="shared" ref="AC17" si="97">AB17/Y17</f>
+      <c r="AF17" s="13">
+        <f t="shared" ref="AF17" si="98">AE17/AB17</f>
         <v>9.3367346938775506E-2</v>
       </c>
-      <c r="AD17" s="4">
-        <f t="shared" ref="AD17" si="98">AB17-AB16</f>
+      <c r="AG17" s="4">
+        <f t="shared" ref="AG17" si="99">AE17-AE16</f>
         <v>46.880000000000109</v>
       </c>
-      <c r="AE17" s="10"/>
-      <c r="AF17" s="8">
-        <f t="shared" ref="AF17" si="99">A17</f>
+      <c r="AH17" s="10"/>
+      <c r="AI17" s="8">
+        <f t="shared" ref="AI17" si="100">A17</f>
         <v>46173</v>
       </c>
-      <c r="AG17" s="4">
-        <f t="shared" ref="AG17" si="100">H17+K17+N17+Q17+T17</f>
+      <c r="AJ17" s="4">
+        <f t="shared" si="15"/>
         <v>1845.3899999999999</v>
       </c>
-      <c r="AH17" s="4">
-        <f t="shared" ref="AH17" si="101">AG17-AG16</f>
+      <c r="AK17" s="4">
+        <f t="shared" ref="AK17" si="101">AJ17-AJ16</f>
         <v>45.389999999999873</v>
       </c>
-      <c r="AI17" s="4">
-        <f t="shared" ref="AI17" si="102">I17+L17+O17+R17+U17</f>
-        <v>2067.35</v>
-      </c>
-      <c r="AJ17" s="4">
-        <f t="shared" ref="AJ17" si="103">AI17-AG17</f>
-        <v>221.96000000000004</v>
-      </c>
-      <c r="AK17" s="13">
-        <f t="shared" ref="AK17" si="104">AJ17/AG17</f>
-        <v>0.12027809839654494</v>
-      </c>
       <c r="AL17" s="4">
-        <f t="shared" ref="AL17" si="105">AJ17-AJ16</f>
+        <f t="shared" si="16"/>
+        <v>2077.35</v>
+      </c>
+      <c r="AM17" s="4">
+        <f t="shared" ref="AM17" si="102">AL17-AJ17</f>
+        <v>231.96000000000004</v>
+      </c>
+      <c r="AN17" s="13">
+        <f t="shared" ref="AN17" si="103">AM17/AJ17</f>
+        <v>0.12569700713670284</v>
+      </c>
+      <c r="AO17" s="4">
+        <f t="shared" ref="AO17" si="104">AM17-AM16</f>
         <v>-6.7799999999999727</v>
       </c>
-      <c r="AM17" s="10"/>
-      <c r="AN17" s="8">
-        <f t="shared" ref="AN17" si="106">A17</f>
+      <c r="AP17" s="10"/>
+      <c r="AQ17" s="8">
+        <f t="shared" ref="AQ17" si="105">A17</f>
         <v>46173</v>
       </c>
-      <c r="AO17" s="4">
-        <f t="shared" ref="AO17" si="107">Y17+AG17</f>
+      <c r="AR17" s="4">
+        <f t="shared" ref="AR17" si="106">AB17+AJ17</f>
         <v>2825.39</v>
       </c>
-      <c r="AP17" s="4">
-        <f t="shared" ref="AP17" si="108">AO17-AO16</f>
+      <c r="AS17" s="4">
+        <f t="shared" ref="AS17" si="107">AR17-AR16</f>
         <v>175.38999999999987</v>
       </c>
-      <c r="AQ17" s="4">
-        <f t="shared" ref="AQ17" si="109">AA17+AI17</f>
-        <v>3138.85</v>
-      </c>
-      <c r="AR17" s="4">
-        <f t="shared" ref="AR17" si="110">AQ17-AO17</f>
-        <v>313.46000000000004</v>
-      </c>
-      <c r="AS17" s="13">
-        <f t="shared" ref="AS17" si="111">AR17/AO17</f>
-        <v>0.1109439758758968</v>
-      </c>
       <c r="AT17" s="4">
-        <f t="shared" ref="AT17" si="112">AR17-AR16</f>
+        <f t="shared" ref="AT17" si="108">AD17+AL17</f>
+        <v>3148.85</v>
+      </c>
+      <c r="AU17" s="4">
+        <f t="shared" ref="AU17" si="109">AT17-AR17</f>
+        <v>323.46000000000004</v>
+      </c>
+      <c r="AV17" s="13">
+        <f t="shared" ref="AV17" si="110">AU17/AR17</f>
+        <v>0.1144833102686709</v>
+      </c>
+      <c r="AW17" s="4">
+        <f t="shared" ref="AW17" si="111">AU17-AU16</f>
         <v>40.100000000000364</v>
       </c>
-      <c r="AV17" s="8">
-        <f t="shared" ref="AV17" si="113">A17</f>
+      <c r="AY17" s="8">
+        <f t="shared" ref="AY17" si="112">A17</f>
         <v>46173</v>
       </c>
-      <c r="AW17" s="4">
-        <f t="shared" ref="AW17" si="114">(C17-B17)-(C16-B16)</f>
+      <c r="AZ17" s="4">
+        <f t="shared" ref="AZ17" si="113">(C17-B17)-(C16-B16)</f>
         <v>20.480000000000075</v>
       </c>
-      <c r="AX17" s="4">
-        <f t="shared" ref="AX17" si="115">(F17-E17)-(F16-E16)</f>
+      <c r="BA17" s="4">
+        <f t="shared" ref="BA17" si="114">(F17-E17)-(F16-E16)</f>
         <v>26.399999999999977</v>
       </c>
-      <c r="AY17" s="4">
-        <f t="shared" ref="AY17" si="116">(I17-H17)-(I16-H16)</f>
+      <c r="BB17" s="4">
+        <f t="shared" ref="BB17" si="115">(I17-H17)-(I16-H16)</f>
         <v>0.25</v>
       </c>
-      <c r="AZ17" s="4">
-        <f t="shared" ref="AZ17" si="117">(L17-K17)-(L16-K16)</f>
+      <c r="BC17" s="4">
+        <f t="shared" ref="BC17" si="116">(L17-K17)-(L16-K16)</f>
         <v>-13.450000000000045</v>
       </c>
-      <c r="BA17" s="4">
-        <f t="shared" ref="BA17" si="118">(O17-N17)-(O16-N16)</f>
+      <c r="BD17" s="4">
+        <f t="shared" ref="BD17" si="117">(O17-N17)-(O16-N16)</f>
         <v>4.3799999999999955</v>
       </c>
-      <c r="BB17" s="4">
-        <f t="shared" ref="BB17" si="119">(R17-Q17)-(R16-Q16)</f>
+      <c r="BE17" s="4">
+        <f t="shared" ref="BE17" si="118">(R17-Q17)-(R16-Q16)</f>
         <v>1.6400000000001</v>
       </c>
-      <c r="BC17" s="4">
-        <f t="shared" ref="BC17" si="120">(U17-T17)-(U16-T16)</f>
+      <c r="BF17" s="4">
+        <f t="shared" si="32"/>
         <v>0.39999999999999858</v>
       </c>
+      <c r="BG17" s="4">
+        <f t="shared" ref="BF17:BG17" si="119">(X17-W17)-(X16-W16)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="18" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>46203</v>
       </c>
@@ -3811,7 +4031,7 @@
         <v>560.79999999999995</v>
       </c>
       <c r="D18" s="11">
-        <f t="shared" ref="D18" si="121">(C18-B18)/B18</f>
+        <f t="shared" ref="D18" si="120">(C18-B18)/B18</f>
         <v>9.9607843137254806E-2</v>
       </c>
       <c r="E18" s="5">
@@ -3821,7 +4041,7 @@
         <v>655.75</v>
       </c>
       <c r="G18" s="11">
-        <f t="shared" ref="G18" si="122">(F18-E18)/E18</f>
+        <f t="shared" ref="G18" si="121">(F18-E18)/E18</f>
         <v>9.2916666666666661E-2</v>
       </c>
       <c r="H18" s="5">
@@ -3831,7 +4051,7 @@
         <v>85.35</v>
       </c>
       <c r="J18" s="12">
-        <f t="shared" ref="J18" si="123">(I18-H18)/H18</f>
+        <f t="shared" ref="J18" si="122">(I18-H18)/H18</f>
         <v>1.8449999999999998</v>
       </c>
       <c r="K18" s="19">
@@ -3841,7 +4061,7 @@
         <v>663.89</v>
       </c>
       <c r="M18" s="12">
-        <f t="shared" ref="M18" si="124">(L18-K18)/K18</f>
+        <f t="shared" ref="M18" si="123">(L18-K18)/K18</f>
         <v>6.3329863057579816E-2</v>
       </c>
       <c r="N18" s="5">
@@ -3851,7 +4071,7 @@
         <v>693.4</v>
       </c>
       <c r="P18" s="12">
-        <f t="shared" ref="P18" si="125">(O18-N18)/N18</f>
+        <f t="shared" ref="P18" si="124">(O18-N18)/N18</f>
         <v>0.11838709677419351</v>
       </c>
       <c r="Q18" s="5">
@@ -3861,7 +4081,7 @@
         <v>667.84</v>
       </c>
       <c r="S18" s="12">
-        <f t="shared" ref="S18" si="126">(R18-Q18)/Q18</f>
+        <f t="shared" ref="S18" si="125">(R18-Q18)/Q18</f>
         <v>9.4819672131147587E-2</v>
       </c>
       <c r="T18" s="5">
@@ -3874,126 +4094,139 @@
         <f>(U18-T18)/T18</f>
         <v>0.16285714285714295</v>
       </c>
-      <c r="X18" s="8">
-        <f t="shared" ref="X18" si="127">A18</f>
+      <c r="W18" s="5">
+        <v>0</v>
+      </c>
+      <c r="X18" s="4">
+        <v>10</v>
+      </c>
+      <c r="Y18" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA18" s="8">
+        <f t="shared" ref="AA18" si="126">A18</f>
         <v>46203</v>
       </c>
-      <c r="Y18" s="4">
-        <f t="shared" ref="Y18" si="128">B18+E18</f>
+      <c r="AB18" s="4">
+        <f t="shared" ref="AB18" si="127">B18+E18</f>
         <v>1110</v>
       </c>
-      <c r="Z18" s="4">
-        <f t="shared" ref="Z18" si="129">Y18-Y17</f>
+      <c r="AC18" s="4">
+        <f t="shared" ref="AC18" si="128">AB18-AB17</f>
         <v>130</v>
       </c>
-      <c r="AA18" s="4">
-        <f t="shared" ref="AA18" si="130">C18+F18</f>
+      <c r="AD18" s="4">
+        <f t="shared" ref="AD18" si="129">C18+F18</f>
         <v>1216.55</v>
       </c>
-      <c r="AB18" s="4">
-        <f t="shared" ref="AB18" si="131">AA18-Y18</f>
+      <c r="AE18" s="4">
+        <f t="shared" ref="AE18" si="130">AD18-AB18</f>
         <v>106.54999999999995</v>
       </c>
-      <c r="AC18" s="13">
-        <f t="shared" ref="AC18" si="132">AB18/Y18</f>
+      <c r="AF18" s="13">
+        <f t="shared" ref="AF18" si="131">AE18/AB18</f>
         <v>9.5990990990990954E-2</v>
       </c>
-      <c r="AD18" s="4">
-        <f t="shared" ref="AD18" si="133">AB18-AB17</f>
+      <c r="AG18" s="4">
+        <f t="shared" ref="AG18" si="132">AE18-AE17</f>
         <v>15.049999999999955</v>
       </c>
-      <c r="AE18" s="10"/>
-      <c r="AF18" s="8">
-        <f t="shared" ref="AF18" si="134">A18</f>
+      <c r="AH18" s="10"/>
+      <c r="AI18" s="8">
+        <f t="shared" ref="AI18" si="133">A18</f>
         <v>46203</v>
       </c>
-      <c r="AG18" s="4">
-        <f t="shared" ref="AG18" si="135">H18+K18+N18+Q18+T18</f>
+      <c r="AJ18" s="4">
+        <f t="shared" si="15"/>
         <v>1954.35</v>
       </c>
-      <c r="AH18" s="4">
-        <f t="shared" ref="AH18" si="136">AG18-AG17</f>
+      <c r="AK18" s="4">
+        <f t="shared" ref="AK18" si="134">AJ18-AJ17</f>
         <v>108.96000000000004</v>
       </c>
-      <c r="AI18" s="4">
-        <f t="shared" ref="AI18" si="137">I18+L18+O18+R18+U18</f>
-        <v>2191.88</v>
-      </c>
-      <c r="AJ18" s="4">
-        <f t="shared" ref="AJ18" si="138">AI18-AG18</f>
-        <v>237.5300000000002</v>
-      </c>
-      <c r="AK18" s="13">
-        <f t="shared" ref="AK18" si="139">AJ18/AG18</f>
-        <v>0.12153913065725187</v>
-      </c>
       <c r="AL18" s="4">
-        <f t="shared" ref="AL18" si="140">AJ18-AJ17</f>
+        <f t="shared" si="16"/>
+        <v>2201.88</v>
+      </c>
+      <c r="AM18" s="4">
+        <f t="shared" ref="AM18" si="135">AL18-AJ18</f>
+        <v>247.5300000000002</v>
+      </c>
+      <c r="AN18" s="13">
+        <f t="shared" ref="AN18" si="136">AM18/AJ18</f>
+        <v>0.12665592140609422</v>
+      </c>
+      <c r="AO18" s="4">
+        <f t="shared" ref="AO18" si="137">AM18-AM17</f>
         <v>15.570000000000164</v>
       </c>
-      <c r="AM18" s="10"/>
-      <c r="AN18" s="8">
-        <f t="shared" ref="AN18" si="141">A18</f>
+      <c r="AP18" s="10"/>
+      <c r="AQ18" s="8">
+        <f t="shared" ref="AQ18" si="138">A18</f>
         <v>46203</v>
       </c>
-      <c r="AO18" s="4">
-        <f t="shared" ref="AO18" si="142">Y18+AG18</f>
+      <c r="AR18" s="4">
+        <f t="shared" ref="AR18" si="139">AB18+AJ18</f>
         <v>3064.35</v>
       </c>
-      <c r="AP18" s="4">
-        <f t="shared" ref="AP18" si="143">AO18-AO17</f>
+      <c r="AS18" s="4">
+        <f t="shared" ref="AS18" si="140">AR18-AR17</f>
         <v>238.96000000000004</v>
       </c>
-      <c r="AQ18" s="4">
-        <f t="shared" ref="AQ18" si="144">AA18+AI18</f>
-        <v>3408.4300000000003</v>
-      </c>
-      <c r="AR18" s="4">
-        <f t="shared" ref="AR18" si="145">AQ18-AO18</f>
-        <v>344.08000000000038</v>
-      </c>
-      <c r="AS18" s="13">
-        <f t="shared" ref="AS18" si="146">AR18/AO18</f>
-        <v>0.11228482386150419</v>
-      </c>
       <c r="AT18" s="4">
-        <f t="shared" ref="AT18" si="147">AR18-AR17</f>
+        <f t="shared" ref="AT18" si="141">AD18+AL18</f>
+        <v>3418.4300000000003</v>
+      </c>
+      <c r="AU18" s="4">
+        <f t="shared" ref="AU18" si="142">AT18-AR18</f>
+        <v>354.08000000000038</v>
+      </c>
+      <c r="AV18" s="13">
+        <f t="shared" ref="AV18" si="143">AU18/AR18</f>
+        <v>0.11554815866333819</v>
+      </c>
+      <c r="AW18" s="4">
+        <f t="shared" ref="AW18" si="144">AU18-AU17</f>
         <v>30.620000000000346</v>
       </c>
-      <c r="AV18" s="8">
-        <f t="shared" ref="AV18" si="148">A18</f>
+      <c r="AY18" s="8">
+        <f t="shared" ref="AY18" si="145">A18</f>
         <v>46203</v>
       </c>
-      <c r="AW18" s="4">
-        <f t="shared" ref="AW18" si="149">(C18-B18)-(C17-B17)</f>
+      <c r="AZ18" s="4">
+        <f t="shared" ref="AZ18" si="146">(C18-B18)-(C17-B17)</f>
         <v>3.7299999999999045</v>
       </c>
-      <c r="AX18" s="4">
-        <f t="shared" ref="AX18" si="150">(F18-E18)-(F17-E17)</f>
+      <c r="BA18" s="4">
+        <f t="shared" ref="BA18" si="147">(F18-E18)-(F17-E17)</f>
         <v>11.32000000000005</v>
       </c>
-      <c r="AY18" s="4">
-        <f t="shared" ref="AY18" si="151">(I18-H18)-(I17-H17)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ18" s="4">
-        <f t="shared" ref="AZ18" si="152">(L18-K18)-(L17-K17)</f>
+      <c r="BB18" s="4">
+        <f t="shared" ref="BB18" si="148">(I18-H18)-(I17-H17)</f>
+        <v>0</v>
+      </c>
+      <c r="BC18" s="4">
+        <f t="shared" ref="BC18" si="149">(L18-K18)-(L17-K17)</f>
         <v>3.75</v>
       </c>
-      <c r="BA18" s="4">
-        <f t="shared" ref="BA18" si="153">(O18-N18)-(O17-N17)</f>
+      <c r="BD18" s="4">
+        <f t="shared" ref="BD18" si="150">(O18-N18)-(O17-N17)</f>
         <v>9.2699999999999818</v>
       </c>
-      <c r="BB18" s="4">
-        <f t="shared" ref="BB18" si="154">(R18-Q18)-(R17-Q17)</f>
+      <c r="BE18" s="4">
+        <f t="shared" ref="BE18" si="151">(R18-Q18)-(R17-Q17)</f>
         <v>1.6499999999999773</v>
       </c>
-      <c r="BC18" s="4">
-        <f t="shared" ref="BC18" si="155">(U18-T18)-(U17-T17)</f>
+      <c r="BF18" s="4">
+        <f t="shared" si="32"/>
         <v>0.90000000000000568</v>
       </c>
+      <c r="BG18" s="4">
+        <f t="shared" ref="BF18:BG18" si="152">(X18-W18)-(X17-W17)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="19" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:59" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>46234</v>
       </c>
@@ -4004,7 +4237,7 @@
         <v>593.07000000000005</v>
       </c>
       <c r="D19" s="11">
-        <f t="shared" ref="D19" si="156">(C19-B19)/B19</f>
+        <f t="shared" ref="D19" si="153">(C19-B19)/B19</f>
         <v>9.8277777777777867E-2</v>
       </c>
       <c r="E19" s="5">
@@ -4014,7 +4247,7 @@
         <v>744.8</v>
       </c>
       <c r="G19" s="11">
-        <f t="shared" ref="G19" si="157">(F19-E19)/E19</f>
+        <f t="shared" ref="G19" si="154">(F19-E19)/E19</f>
         <v>6.3999999999999932E-2</v>
       </c>
       <c r="H19" s="5">
@@ -4024,7 +4257,7 @@
         <v>85.35</v>
       </c>
       <c r="J19" s="12">
-        <f t="shared" ref="J19" si="158">(I19-H19)/H19</f>
+        <f t="shared" ref="J19" si="155">(I19-H19)/H19</f>
         <v>1.8449999999999998</v>
       </c>
       <c r="K19" s="19">
@@ -4034,7 +4267,7 @@
         <v>666.13</v>
       </c>
       <c r="M19" s="12">
-        <f t="shared" ref="M19" si="159">(L19-K19)/K19</f>
+        <f t="shared" ref="M19" si="156">(L19-K19)/K19</f>
         <v>6.6917594298069941E-2</v>
       </c>
       <c r="N19" s="5">
@@ -4044,7 +4277,7 @@
         <v>695.94</v>
       </c>
       <c r="P19" s="12">
-        <f t="shared" ref="P19" si="160">(O19-N19)/N19</f>
+        <f t="shared" ref="P19" si="157">(O19-N19)/N19</f>
         <v>0.12248387096774202</v>
       </c>
       <c r="Q19" s="5">
@@ -4054,7 +4287,7 @@
         <v>669.6</v>
       </c>
       <c r="S19" s="12">
-        <f t="shared" ref="S19" si="161">(R19-Q19)/Q19</f>
+        <f t="shared" ref="S19" si="158">(R19-Q19)/Q19</f>
         <v>9.7704918032786928E-2</v>
       </c>
       <c r="T19" s="5">
@@ -4067,145 +4300,159 @@
         <f>(U19-T19)/T19</f>
         <v>0.17285714285714276</v>
       </c>
-      <c r="X19" s="8">
-        <f t="shared" ref="X19" si="162">A19</f>
+      <c r="W19" s="5">
+        <v>0</v>
+      </c>
+      <c r="X19" s="4">
+        <v>10</v>
+      </c>
+      <c r="Y19" s="12">
+        <v>0</v>
+      </c>
+      <c r="AA19" s="8">
+        <f t="shared" ref="AA19" si="159">A19</f>
         <v>46234</v>
       </c>
-      <c r="Y19" s="4">
-        <f t="shared" ref="Y19" si="163">B19+E19</f>
+      <c r="AB19" s="4">
+        <f t="shared" ref="AB19" si="160">B19+E19</f>
         <v>1240</v>
       </c>
-      <c r="Z19" s="4">
-        <f t="shared" ref="Z19" si="164">Y19-Y18</f>
+      <c r="AC19" s="4">
+        <f t="shared" ref="AC19" si="161">AB19-AB18</f>
         <v>130</v>
       </c>
-      <c r="AA19" s="4">
-        <f t="shared" ref="AA19" si="165">C19+F19</f>
+      <c r="AD19" s="4">
+        <f t="shared" ref="AD19" si="162">C19+F19</f>
         <v>1337.87</v>
       </c>
-      <c r="AB19" s="4">
-        <f t="shared" ref="AB19" si="166">AA19-Y19</f>
+      <c r="AE19" s="4">
+        <f t="shared" ref="AE19" si="163">AD19-AB19</f>
         <v>97.869999999999891</v>
       </c>
-      <c r="AC19" s="13">
-        <f t="shared" ref="AC19" si="167">AB19/Y19</f>
+      <c r="AF19" s="13">
+        <f t="shared" ref="AF19" si="164">AE19/AB19</f>
         <v>7.8927419354838615E-2</v>
       </c>
-      <c r="AD19" s="4">
-        <f t="shared" ref="AD19" si="168">AB19-AB18</f>
+      <c r="AG19" s="4">
+        <f t="shared" ref="AG19" si="165">AE19-AE18</f>
         <v>-8.6800000000000637</v>
       </c>
-      <c r="AE19" s="10"/>
-      <c r="AF19" s="8">
-        <f t="shared" ref="AF19" si="169">A19</f>
+      <c r="AH19" s="10"/>
+      <c r="AI19" s="8">
+        <f t="shared" ref="AI19" si="166">A19</f>
         <v>46234</v>
       </c>
-      <c r="AG19" s="4">
-        <f t="shared" ref="AG19" si="170">H19+K19+N19+Q19+T19</f>
+      <c r="AJ19" s="4">
+        <f t="shared" si="15"/>
         <v>1954.35</v>
       </c>
-      <c r="AH19" s="4">
-        <f t="shared" ref="AH19" si="171">AG19-AG18</f>
-        <v>0</v>
-      </c>
-      <c r="AI19" s="4">
-        <f>I19+L19+O19+R19+U19</f>
-        <v>2199.12</v>
-      </c>
-      <c r="AJ19" s="4">
-        <f t="shared" ref="AJ19" si="172">AI19-AG19</f>
-        <v>244.76999999999998</v>
-      </c>
-      <c r="AK19" s="13">
-        <f t="shared" ref="AK19" si="173">AJ19/AG19</f>
-        <v>0.12524368715941361</v>
+      <c r="AK19" s="4">
+        <f t="shared" ref="AK19" si="167">AJ19-AJ18</f>
+        <v>0</v>
       </c>
       <c r="AL19" s="4">
-        <f t="shared" ref="AL19" si="174">AJ19-AJ18</f>
+        <f t="shared" si="16"/>
+        <v>2209.12</v>
+      </c>
+      <c r="AM19" s="4">
+        <f t="shared" ref="AM19" si="168">AL19-AJ19</f>
+        <v>254.76999999999998</v>
+      </c>
+      <c r="AN19" s="13">
+        <f t="shared" ref="AN19" si="169">AM19/AJ19</f>
+        <v>0.13036047790825595</v>
+      </c>
+      <c r="AO19" s="4">
+        <f t="shared" ref="AO19" si="170">AM19-AM18</f>
         <v>7.2399999999997817</v>
       </c>
-      <c r="AM19" s="10"/>
-      <c r="AN19" s="8">
-        <f t="shared" ref="AN19" si="175">A19</f>
+      <c r="AP19" s="10"/>
+      <c r="AQ19" s="8">
+        <f t="shared" ref="AQ19" si="171">A19</f>
         <v>46234</v>
       </c>
-      <c r="AO19" s="4">
-        <f t="shared" ref="AO19" si="176">Y19+AG19</f>
+      <c r="AR19" s="4">
+        <f t="shared" ref="AR19" si="172">AB19+AJ19</f>
         <v>3194.35</v>
       </c>
-      <c r="AP19" s="4">
-        <f t="shared" ref="AP19" si="177">AO19-AO18</f>
+      <c r="AS19" s="4">
+        <f t="shared" ref="AS19" si="173">AR19-AR18</f>
         <v>130</v>
       </c>
-      <c r="AQ19" s="4">
-        <f t="shared" ref="AQ19" si="178">AA19+AI19</f>
-        <v>3536.99</v>
-      </c>
-      <c r="AR19" s="4">
-        <f t="shared" ref="AR19" si="179">AQ19-AO19</f>
-        <v>342.63999999999987</v>
-      </c>
-      <c r="AS19" s="13">
-        <f t="shared" ref="AS19" si="180">AR19/AO19</f>
-        <v>0.10726438868627416</v>
-      </c>
       <c r="AT19" s="4">
-        <f t="shared" ref="AT19" si="181">AR19-AR18</f>
+        <f t="shared" ref="AT19" si="174">AD19+AL19</f>
+        <v>3546.99</v>
+      </c>
+      <c r="AU19" s="4">
+        <f t="shared" ref="AU19" si="175">AT19-AR19</f>
+        <v>352.63999999999987</v>
+      </c>
+      <c r="AV19" s="13">
+        <f t="shared" ref="AV19" si="176">AU19/AR19</f>
+        <v>0.11039491602360414</v>
+      </c>
+      <c r="AW19" s="4">
+        <f t="shared" ref="AW19" si="177">AU19-AU18</f>
         <v>-1.4400000000005093</v>
       </c>
-      <c r="AV19" s="8">
-        <f t="shared" ref="AV19" si="182">A19</f>
+      <c r="AY19" s="8">
+        <f t="shared" ref="AY19" si="178">A19</f>
         <v>46234</v>
       </c>
-      <c r="AW19" s="4">
-        <f t="shared" ref="AW19" si="183">(C19-B19)-(C18-B18)</f>
+      <c r="AZ19" s="4">
+        <f t="shared" ref="AZ19" si="179">(C19-B19)-(C18-B18)</f>
         <v>2.2700000000000955</v>
       </c>
-      <c r="AX19" s="4">
-        <f t="shared" ref="AX19" si="184">(F19-E19)-(F18-E18)</f>
+      <c r="BA19" s="4">
+        <f t="shared" ref="BA19" si="180">(F19-E19)-(F18-E18)</f>
         <v>-10.950000000000045</v>
       </c>
-      <c r="AY19" s="4">
-        <f t="shared" ref="AY19" si="185">(I19-H19)-(I18-H18)</f>
-        <v>0</v>
-      </c>
-      <c r="AZ19" s="4">
-        <f t="shared" ref="AZ19" si="186">(L19-K19)-(L18-K18)</f>
+      <c r="BB19" s="4">
+        <f t="shared" ref="BB19" si="181">(I19-H19)-(I18-H18)</f>
+        <v>0</v>
+      </c>
+      <c r="BC19" s="4">
+        <f t="shared" ref="BC19" si="182">(L19-K19)-(L18-K18)</f>
         <v>2.2400000000000091</v>
       </c>
-      <c r="BA19" s="4">
-        <f t="shared" ref="BA19" si="187">(O19-N19)-(O18-N18)</f>
+      <c r="BD19" s="4">
+        <f t="shared" ref="BD19" si="183">(O19-N19)-(O18-N18)</f>
         <v>2.5400000000000773</v>
       </c>
-      <c r="BB19" s="4">
-        <f t="shared" ref="BB19" si="188">(R19-Q19)-(R18-Q18)</f>
+      <c r="BE19" s="4">
+        <f t="shared" ref="BE19" si="184">(R19-Q19)-(R18-Q18)</f>
         <v>1.7599999999999909</v>
       </c>
-      <c r="BC19" s="4">
-        <f t="shared" ref="BC19" si="189">(U19-T19)-(U18-T18)</f>
+      <c r="BF19" s="4">
+        <f t="shared" si="32"/>
         <v>0.69999999999998863</v>
+      </c>
+      <c r="BG19" s="4">
+        <f t="shared" ref="BF19:BG19" si="185">(X19-W19)-(X18-W18)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="AV1:BC1"/>
+  <mergeCells count="13">
+    <mergeCell ref="AY1:BG1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="E1:G1"/>
-    <mergeCell ref="X1:AD1"/>
+    <mergeCell ref="AA1:AG1"/>
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="Q1:S1"/>
+    <mergeCell ref="W1:Y1"/>
+    <mergeCell ref="AI1:AO1"/>
+    <mergeCell ref="AQ1:AW1"/>
     <mergeCell ref="T1:V1"/>
-    <mergeCell ref="AF1:AL1"/>
-    <mergeCell ref="AN1:AT1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="AP3:AP19" formula="1"/>
+    <ignoredError sqref="AS3:AS19" formula="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Dashboard update 2026-08-07 22:21
</commit_message>
<xml_diff>
--- a/excel/Investavimas Rima.xlsx
+++ b/excel/Investavimas Rima.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evald\OneDrive\Dokumentai\portfolio-analytics\portfolio-dashboard-clean\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5E43EB3-8976-4462-B2F3-D895F46CAB2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34D7C101-0694-407F-A03B-561C9EE974C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4534,19 +4534,19 @@
         <v>0.17285714285714276</v>
       </c>
       <c r="W19" s="5">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="X19" s="4">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="Y19" s="12">
         <v>0</v>
       </c>
       <c r="Z19" s="5">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="AA19" s="4">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AB19" s="12">
         <v>0</v>
@@ -4586,27 +4586,27 @@
       </c>
       <c r="AM19" s="4">
         <f>H19+K19+N19+Q19+T19+W19+Z19</f>
-        <v>1975.35</v>
+        <v>1954.35</v>
       </c>
       <c r="AN19" s="4">
         <f t="shared" ref="AN19" si="168">AM19-AM18</f>
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="AO19" s="4">
         <f>I19+L19+O19+R19+U19+X19+AA19</f>
-        <v>2222.12</v>
+        <v>2199.12</v>
       </c>
       <c r="AP19" s="4">
         <f t="shared" ref="AP19" si="169">AO19-AM19</f>
-        <v>246.76999999999998</v>
+        <v>244.76999999999998</v>
       </c>
       <c r="AQ19" s="13">
         <f t="shared" ref="AQ19" si="170">AP19/AM19</f>
-        <v>0.12492469688915887</v>
+        <v>0.12524368715941361</v>
       </c>
       <c r="AR19" s="4">
         <f t="shared" ref="AR19" si="171">AP19-AP18</f>
-        <v>9.2399999999997817</v>
+        <v>7.2399999999997817</v>
       </c>
       <c r="AS19" s="10"/>
       <c r="AT19" s="8">
@@ -4615,27 +4615,27 @@
       </c>
       <c r="AU19" s="4">
         <f t="shared" ref="AU19" si="173">AE19+AM19</f>
-        <v>3215.35</v>
+        <v>3194.35</v>
       </c>
       <c r="AV19" s="4">
         <f t="shared" ref="AV19" si="174">AU19-AU18</f>
-        <v>151</v>
+        <v>130</v>
       </c>
       <c r="AW19" s="4">
         <f t="shared" ref="AW19" si="175">AG19+AO19</f>
-        <v>3559.99</v>
+        <v>3536.99</v>
       </c>
       <c r="AX19" s="4">
         <f t="shared" ref="AX19" si="176">AW19-AU19</f>
-        <v>344.63999999999987</v>
+        <v>342.63999999999987</v>
       </c>
       <c r="AY19" s="13">
         <f t="shared" ref="AY19" si="177">AX19/AU19</f>
-        <v>0.10718584290979205</v>
+        <v>0.10726438868627416</v>
       </c>
       <c r="AZ19" s="4">
         <f t="shared" ref="AZ19" si="178">AX19-AX18</f>
-        <v>0.55999999999949068</v>
+        <v>-1.4400000000005093</v>
       </c>
       <c r="BB19" s="8">
         <f t="shared" ref="BB19" si="179">A19</f>
@@ -4671,11 +4671,11 @@
       </c>
       <c r="BJ19" s="4">
         <f t="shared" si="33"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BK19" s="4">
         <f t="shared" ref="BK19" si="186">(AA19-Z19)-(AA18-Z18)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>